<commit_message>
docs: register refresh, KT-STD-001 v1.9, PRC-CHG-001 drafts, Tenders v0.12 working copy
- Baseline register and documentation control register refreshed for the
  current document set.
- KenTender_KT-STD-001 v1.9 (Document Design and Verification Standards).
- New 13_proceedings: PRC-CHG-001 Minimal Procurement Proceedings v0.1 and
  v0.2, with the functional design source.
- Tenders working copy moves to v0.12; the superseded v0.11 working copy is
  removed (kept in history).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/mvp-1-r1/98_work_progress/KenTender_Documentation_Control_Register.xlsx
+++ b/docs/mvp-1-r1/98_work_progress/KenTender_Documentation_Control_Register.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R004619dfe2d948a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="2" r:id="Rf11418edcc5f4afa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interfaces" sheetId="3" r:id="Rbaad753d0f1d4af1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Rf0296969abad41d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery" sheetId="5" r:id="R1b1e76033e814cf7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future Work" sheetId="6" r:id="Rbe951852b697406e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="7" r:id="R06ef8e1c7579449f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf03793996ed843ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="2" r:id="R40d4e62b43384dac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interfaces" sheetId="3" r:id="R5c340d2232684845"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R9364b9ae0d004b12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery" sheetId="5" r:id="R264f413469df47da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future Work" sheetId="6" r:id="R7ea02c27ad7848be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="7" r:id="R0bda82e023d34079"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -252,7 +252,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -263,7 +263,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -274,7 +274,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -285,7 +285,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -296,7 +296,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -307,7 +307,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -317,7 +317,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -328,7 +328,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -339,7 +339,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -349,7 +349,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -359,7 +359,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -370,7 +370,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -381,7 +381,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -392,7 +392,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -403,7 +403,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -413,7 +413,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -424,7 +424,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -435,7 +435,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -445,7 +445,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -455,7 +455,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -466,7 +466,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -477,7 +477,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -488,7 +488,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -499,7 +499,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -509,7 +509,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -520,7 +520,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -531,7 +531,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -541,7 +541,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -551,7 +551,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -562,7 +562,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -573,7 +573,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -584,7 +584,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -595,7 +595,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -605,7 +605,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -616,7 +616,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -627,7 +627,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -637,7 +637,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -647,7 +647,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -658,7 +658,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -669,7 +669,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -680,7 +680,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -691,7 +691,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -701,7 +701,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -712,7 +712,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -723,7 +723,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -733,7 +733,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -743,7 +743,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -754,7 +754,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -765,7 +765,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -776,7 +776,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -787,7 +787,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -797,7 +797,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -808,7 +808,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -819,7 +819,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -829,7 +829,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -839,7 +839,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -850,7 +850,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -861,7 +861,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -872,7 +872,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -883,7 +883,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -893,7 +893,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -904,7 +904,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -915,7 +915,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -925,7 +925,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -935,7 +935,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -946,7 +946,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -957,7 +957,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -968,7 +968,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -979,7 +979,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -989,7 +989,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -1000,7 +1000,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -1011,7 +1011,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -1021,7 +1021,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -1031,7 +1031,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -1042,7 +1042,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -1053,7 +1053,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -1064,7 +1064,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -1075,7 +1075,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -1085,7 +1085,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -1096,7 +1096,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -1107,7 +1107,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -1117,7 +1117,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -1127,7 +1127,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -1138,7 +1138,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -1149,7 +1149,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -1160,7 +1160,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -1171,7 +1171,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -1181,7 +1181,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -1192,7 +1192,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -1203,7 +1203,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -1213,7 +1213,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -1223,7 +1223,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -1234,7 +1234,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -1245,7 +1245,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -1256,7 +1256,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -1267,7 +1267,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -1277,7 +1277,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -1288,7 +1288,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -1299,7 +1299,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -1309,7 +1309,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -1319,7 +1319,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -1330,7 +1330,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -1341,7 +1341,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -1352,7 +1352,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -1363,7 +1363,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -1373,7 +1373,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -1384,7 +1384,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -1395,7 +1395,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -1405,7 +1405,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -1415,7 +1415,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -1426,7 +1426,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -1437,7 +1437,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -1448,7 +1448,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -1459,7 +1459,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -1469,7 +1469,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -1480,7 +1480,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -1491,7 +1491,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -1501,7 +1501,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -1511,7 +1511,7 @@
         <x:color rgb="FF1F2937"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFF2F2F2"/>
         </x:patternFill>
       </x:fill>
@@ -1522,7 +1522,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -1533,7 +1533,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -1586,8 +1586,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DecisionsTable" displayName="DecisionsTable" ref="A5:F28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:F28"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DecisionsTable" displayName="DecisionsTable" ref="A5:F29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:F29"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Decision ID"/>
     <x:tableColumn id="2" name="Decision"/>
@@ -1894,7 +1894,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>Current controlled baseline and delivery status as at 2026-09-25. Requirement approval, implementation, verification and release are tracked independently.</x:v>
+        <x:v>Current controlled baseline and delivery status as at 2026-09-26. Requirement approval, implementation, verification and release are tracked independently.</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -2024,12 +2024,12 @@
       <x:c r="B6" s="20"/>
       <x:c r="C6" s="20" t="n">
         <x:f>COUNTIF(Documents!F6:F29,"Approved requirement")</x:f>
-        <x:v>8</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D6" s="20"/>
       <x:c r="E6" s="20" t="n">
         <x:f>COUNTIF(Documents!F6:F29,"Project Owner review")</x:f>
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="F6" s="20"/>
       <x:c r="G6" s="20" t="n">
@@ -2186,7 +2186,7 @@
       <x:c r="Y10" s="2"/>
       <x:c r="Z10" s="2"/>
     </x:row>
-    <x:row r="11" ht="48" customHeight="1">
+    <x:row r="11" ht="24" hidden="0" customHeight="1">
       <x:c r="A11" s="24" t="str">
         <x:v>AUD-001</x:v>
       </x:c>
@@ -2230,7 +2230,7 @@
       <x:c r="Y11" s="2"/>
       <x:c r="Z11" s="2"/>
     </x:row>
-    <x:row r="12" ht="48" customHeight="1">
+    <x:row r="12" ht="42" hidden="0" customHeight="1">
       <x:c r="A12" s="24" t="str">
         <x:v>AUD-002</x:v>
       </x:c>
@@ -2241,7 +2241,7 @@
         <x:v>Approval</x:v>
       </x:c>
       <x:c r="D12" s="24" t="str">
-        <x:v>Complete final cross-document review and approve.</x:v>
+        <x:v>No approval action remains; implementation and verification are tracked separately.</x:v>
       </x:c>
       <x:c r="E12" s="24" t="str">
         <x:v>Project Owner</x:v>
@@ -2250,10 +2250,10 @@
         <x:v>Authoritative Tender implementation baseline</x:v>
       </x:c>
       <x:c r="G12" s="24" t="str">
-        <x:v>Open</x:v>
+        <x:v>Closed</x:v>
       </x:c>
       <x:c r="H12" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.11 control block</x:v>
+        <x:v>TPR-CHG-001 v0.12 approval control block</x:v>
       </x:c>
       <x:c r="I12" s="2"/>
       <x:c r="J12" s="2"/>
@@ -2274,7 +2274,7 @@
       <x:c r="Y12" s="2"/>
       <x:c r="Z12" s="2"/>
     </x:row>
-    <x:row r="13" ht="48" customHeight="1">
+    <x:row r="13" ht="24" hidden="0" customHeight="1">
       <x:c r="A13" s="24" t="str">
         <x:v>AUD-003</x:v>
       </x:c>
@@ -2285,19 +2285,19 @@
         <x:v>Approval</x:v>
       </x:c>
       <x:c r="D13" s="24" t="str">
-        <x:v>Approve after Gate 1 reconciliation.</x:v>
+        <x:v>No further requirement approval for v0.8; retain separate TPR v0.13 dependency and production operating gates.</x:v>
       </x:c>
       <x:c r="E13" s="24" t="str">
         <x:v>Project Owner</x:v>
       </x:c>
       <x:c r="F13" s="24" t="str">
-        <x:v>Authoritative Bid Submission implementation baseline</x:v>
+        <x:v>None—requirements approval recorded</x:v>
       </x:c>
       <x:c r="G13" s="24" t="str">
-        <x:v>Open</x:v>
+        <x:v>Closed</x:v>
       </x:c>
       <x:c r="H13" s="24" t="str">
-        <x:v>BDS-CHG-001 v0.7 control block</x:v>
+        <x:v>BDS-CHG-001 v0.8 approval record</x:v>
       </x:c>
       <x:c r="I13" s="2"/>
       <x:c r="J13" s="2"/>
@@ -2318,9 +2318,9 @@
       <x:c r="Y13" s="2"/>
       <x:c r="Z13" s="2"/>
     </x:row>
-    <x:row r="14" ht="48" customHeight="1">
+    <x:row r="14" ht="24" hidden="0" customHeight="1">
       <x:c r="A14" s="24" t="str">
-        <x:v>AUD-004</x:v>
+        <x:v>AUD-005</x:v>
       </x:c>
       <x:c r="B14" s="24" t="str">
         <x:v>High</x:v>
@@ -2329,19 +2329,19 @@
         <x:v>Approval</x:v>
       </x:c>
       <x:c r="D14" s="24" t="str">
-        <x:v>Approve curation and release standard.</x:v>
+        <x:v>Approve as the current Gate 1 delivery control.</x:v>
       </x:c>
       <x:c r="E14" s="24" t="str">
         <x:v>Project Owner</x:v>
       </x:c>
       <x:c r="F14" s="24" t="str">
-        <x:v>Rebuilt response-capable tender bundle</x:v>
+        <x:v>Single authoritative change matrix</x:v>
       </x:c>
       <x:c r="G14" s="24" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H14" s="24" t="str">
-        <x:v>STD-TPL-001 v0.10 control block</x:v>
+        <x:v>G1-REG-001 v1.1 control block</x:v>
       </x:c>
       <x:c r="I14" s="2"/>
       <x:c r="J14" s="2"/>
@@ -2362,30 +2362,30 @@
       <x:c r="Y14" s="2"/>
       <x:c r="Z14" s="2"/>
     </x:row>
-    <x:row r="15" ht="48" customHeight="1">
+    <x:row r="15" ht="48.75" hidden="0" customHeight="1">
       <x:c r="A15" s="24" t="str">
-        <x:v>AUD-005</x:v>
+        <x:v>AUD-006</x:v>
       </x:c>
       <x:c r="B15" s="24" t="str">
-        <x:v>High</x:v>
+        <x:v>Critical</x:v>
       </x:c>
       <x:c r="C15" s="24" t="str">
-        <x:v>Approval</x:v>
+        <x:v>Bundle readiness</x:v>
       </x:c>
       <x:c r="D15" s="24" t="str">
-        <x:v>Approve as the current Gate 1 delivery control.</x:v>
+        <x:v>Rebuild and verify the bundle; install with matching assets and renderer, then Administrator may turn it On.</x:v>
       </x:c>
       <x:c r="E15" s="24" t="str">
-        <x:v>Project Owner</x:v>
+        <x:v>Controlled release owner</x:v>
       </x:c>
       <x:c r="F15" s="24" t="str">
-        <x:v>Single authoritative change matrix</x:v>
+        <x:v>Tender publication and production Bid Submission</x:v>
       </x:c>
       <x:c r="G15" s="24" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H15" s="24" t="str">
-        <x:v>G1-REG-001 v1.1 control block</x:v>
+        <x:v>STD-TPL-001 v0.10 in-version amendment; FU-01 OD5; earlier candidate ZIP</x:v>
       </x:c>
       <x:c r="I15" s="2"/>
       <x:c r="J15" s="2"/>
@@ -2406,30 +2406,30 @@
       <x:c r="Y15" s="2"/>
       <x:c r="Z15" s="2"/>
     </x:row>
-    <x:row r="16" ht="48" customHeight="1">
+    <x:row r="16" ht="66" hidden="0" customHeight="1">
       <x:c r="A16" s="24" t="str">
-        <x:v>AUD-006</x:v>
+        <x:v>AUD-007</x:v>
       </x:c>
       <x:c r="B16" s="24" t="str">
         <x:v>Critical</x:v>
       </x:c>
       <x:c r="C16" s="24" t="str">
-        <x:v>Release gate</x:v>
+        <x:v>Operating gate</x:v>
       </x:c>
       <x:c r="D16" s="24" t="str">
-        <x:v>Rebuild, verify and approve the exact manifest.</x:v>
+        <x:v>Approve support, monitoring, recovery, authority and incident arrangements; then enable the deployment flag.</x:v>
       </x:c>
       <x:c r="E16" s="24" t="str">
-        <x:v>Controlled release owner</x:v>
+        <x:v>Project Owner / Operations</x:v>
       </x:c>
       <x:c r="F16" s="24" t="str">
-        <x:v>Tender publication and production Bid Submission</x:v>
+        <x:v>Production submission</x:v>
       </x:c>
       <x:c r="G16" s="24" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H16" s="24" t="str">
-        <x:v>STD-TPL-001 v0.10; candidate ZIP</x:v>
+        <x:v>BDS-CHG-001 v0.8; G1-REG-001 v1.1</x:v>
       </x:c>
       <x:c r="I16" s="2"/>
       <x:c r="J16" s="2"/>
@@ -2450,30 +2450,30 @@
       <x:c r="Y16" s="2"/>
       <x:c r="Z16" s="2"/>
     </x:row>
-    <x:row r="17" ht="48" customHeight="1">
+    <x:row r="17" ht="48.75" hidden="0" customHeight="1">
       <x:c r="A17" s="24" t="str">
-        <x:v>AUD-007</x:v>
+        <x:v>AUD-008</x:v>
       </x:c>
       <x:c r="B17" s="24" t="str">
-        <x:v>Critical</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="C17" s="24" t="str">
-        <x:v>Operating gate</x:v>
+        <x:v>Reconciliation</x:v>
       </x:c>
       <x:c r="D17" s="24" t="str">
-        <x:v>Approve support, monitoring, recovery, authority and incident arrangements; then enable the deployment flag.</x:v>
+        <x:v>Issue a reconciled fixture version before integrated verification.</x:v>
       </x:c>
       <x:c r="E17" s="24" t="str">
-        <x:v>Project Owner / Operations</x:v>
+        <x:v>Requirements owner</x:v>
       </x:c>
       <x:c r="F17" s="24" t="str">
-        <x:v>Production submission</x:v>
+        <x:v>Reliable end-to-end seed tests</x:v>
       </x:c>
       <x:c r="G17" s="24" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H17" s="24" t="str">
-        <x:v>BDS-CHG-001 v0.7; G1-REG-001 v1.1</x:v>
+        <x:v>SEED-001 v1.3 compared with current baseline</x:v>
       </x:c>
       <x:c r="I17" s="2"/>
       <x:c r="J17" s="2"/>
@@ -2494,30 +2494,30 @@
       <x:c r="Y17" s="2"/>
       <x:c r="Z17" s="2"/>
     </x:row>
-    <x:row r="18" ht="48" customHeight="1">
+    <x:row r="18" ht="45" hidden="0" customHeight="1">
       <x:c r="A18" s="24" t="str">
-        <x:v>AUD-008</x:v>
+        <x:v>AUD-009</x:v>
       </x:c>
       <x:c r="B18" s="24" t="str">
-        <x:v>High</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="C18" s="24" t="str">
-        <x:v>Reconciliation</x:v>
+        <x:v>Stale reference</x:v>
       </x:c>
       <x:c r="D18" s="24" t="str">
-        <x:v>Issue a reconciled fixture version before integrated verification.</x:v>
+        <x:v>Refresh document references without changing the approved legal decision.</x:v>
       </x:c>
       <x:c r="E18" s="24" t="str">
         <x:v>Requirements owner</x:v>
       </x:c>
       <x:c r="F18" s="24" t="str">
-        <x:v>Reliable end-to-end seed tests</x:v>
+        <x:v>Clean reservation implementation handoff</x:v>
       </x:c>
       <x:c r="G18" s="24" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H18" s="24" t="str">
-        <x:v>SEED-001 v1.3 compared with current baseline</x:v>
+        <x:v>RES-IMP-001 v1.0 references</x:v>
       </x:c>
       <x:c r="I18" s="2"/>
       <x:c r="J18" s="2"/>
@@ -2538,30 +2538,30 @@
       <x:c r="Y18" s="2"/>
       <x:c r="Z18" s="2"/>
     </x:row>
-    <x:row r="19" ht="48" customHeight="1">
+    <x:row r="19" ht="45" hidden="0" customHeight="1">
       <x:c r="A19" s="24" t="str">
-        <x:v>AUD-009</x:v>
+        <x:v>AUD-010</x:v>
       </x:c>
       <x:c r="B19" s="24" t="str">
-        <x:v>Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="C19" s="24" t="str">
-        <x:v>Stale reference</x:v>
+        <x:v>Missing controlled file</x:v>
       </x:c>
       <x:c r="D19" s="24" t="str">
-        <x:v>Refresh document references without changing the approved legal decision.</x:v>
+        <x:v>Locate or admit the exact version and record its authority.</x:v>
       </x:c>
       <x:c r="E19" s="24" t="str">
-        <x:v>Requirements owner</x:v>
+        <x:v>Documentation owner</x:v>
       </x:c>
       <x:c r="F19" s="24" t="str">
-        <x:v>Clean reservation implementation handoff</x:v>
+        <x:v>Complete template/tender/bid traceability</x:v>
       </x:c>
       <x:c r="G19" s="24" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H19" s="24" t="str">
-        <x:v>RES-IMP-001 v1.0 references</x:v>
+        <x:v>References in current controlled documents</x:v>
       </x:c>
       <x:c r="I19" s="2"/>
       <x:c r="J19" s="2"/>
@@ -2582,9 +2582,9 @@
       <x:c r="Y19" s="2"/>
       <x:c r="Z19" s="2"/>
     </x:row>
-    <x:row r="20" ht="48" customHeight="1">
+    <x:row r="20" ht="42" hidden="0" customHeight="1">
       <x:c r="A20" s="24" t="str">
-        <x:v>AUD-010</x:v>
+        <x:v>AUD-011</x:v>
       </x:c>
       <x:c r="B20" s="24" t="str">
         <x:v>High</x:v>
@@ -2593,13 +2593,13 @@
         <x:v>Missing controlled file</x:v>
       </x:c>
       <x:c r="D20" s="24" t="str">
-        <x:v>Locate or admit the exact version and record its authority.</x:v>
+        <x:v>Locate or admit the exact version before integrated stress testing.</x:v>
       </x:c>
       <x:c r="E20" s="24" t="str">
         <x:v>Documentation owner</x:v>
       </x:c>
       <x:c r="F20" s="24" t="str">
-        <x:v>Complete template/tender/bid traceability</x:v>
+        <x:v>Gate 1 integrated verification</x:v>
       </x:c>
       <x:c r="G20" s="24" t="str">
         <x:v>Open</x:v>
@@ -2626,30 +2626,30 @@
       <x:c r="Y20" s="2"/>
       <x:c r="Z20" s="2"/>
     </x:row>
-    <x:row r="21" ht="48" customHeight="1">
+    <x:row r="21" ht="55.5" hidden="0" customHeight="1">
       <x:c r="A21" s="24" t="str">
-        <x:v>AUD-011</x:v>
+        <x:v>AUD-013</x:v>
       </x:c>
       <x:c r="B21" s="24" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="C21" s="24" t="str">
-        <x:v>Missing controlled file</x:v>
+        <x:v>Cross-module adoption</x:v>
       </x:c>
       <x:c r="D21" s="24" t="str">
-        <x:v>Locate or admit the exact version before integrated stress testing.</x:v>
+        <x:v>Adopt the shared contract in each active module and run persona/state conformance tests.</x:v>
       </x:c>
       <x:c r="E21" s="24" t="str">
-        <x:v>Documentation owner</x:v>
+        <x:v>Requirements and implementation owners</x:v>
       </x:c>
       <x:c r="F21" s="24" t="str">
-        <x:v>Gate 1 integrated verification</x:v>
+        <x:v>Usability-complete Gate 1 verification</x:v>
       </x:c>
       <x:c r="G21" s="24" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H21" s="24" t="str">
-        <x:v>References in current controlled documents</x:v>
+        <x:v>KT-STD-001 v1.9; PLN-CHG-001 v1.27; Workflow Guidance Standard</x:v>
       </x:c>
       <x:c r="I21" s="2"/>
       <x:c r="J21" s="2"/>
@@ -2670,30 +2670,30 @@
       <x:c r="Y21" s="2"/>
       <x:c r="Z21" s="2"/>
     </x:row>
-    <x:row r="22" ht="48" customHeight="1">
+    <x:row r="22" ht="48.75" hidden="0" customHeight="1">
       <x:c r="A22" s="24" t="str">
-        <x:v>AUD-013</x:v>
+        <x:v>AUD-014</x:v>
       </x:c>
       <x:c r="B22" s="24" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="C22" s="24" t="str">
-        <x:v>Cross-module adoption</x:v>
+        <x:v>Implementation handoff</x:v>
       </x:c>
       <x:c r="D22" s="24" t="str">
-        <x:v>Adopt the shared contract in each active module and run persona/state conformance tests.</x:v>
+        <x:v>Issue a controlled SEED successor before integrated implementation verification.</x:v>
       </x:c>
       <x:c r="E22" s="24" t="str">
-        <x:v>Requirements and implementation owners</x:v>
+        <x:v>Requirements owner</x:v>
       </x:c>
       <x:c r="F22" s="24" t="str">
-        <x:v>Usability-complete Gate 1 verification</x:v>
+        <x:v>One reproducible end-to-end test baseline</x:v>
       </x:c>
       <x:c r="G22" s="24" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H22" s="24" t="str">
-        <x:v>KT-STD-001 v1.8; PLN-CHG-001 v1.27; Workflow Guidance Standard</x:v>
+        <x:v>G1-REG-001 v1.1; SEED-001 v1.3 compared with current baseline</x:v>
       </x:c>
       <x:c r="I22" s="2"/>
       <x:c r="J22" s="2"/>
@@ -2714,30 +2714,30 @@
       <x:c r="Y22" s="2"/>
       <x:c r="Z22" s="2"/>
     </x:row>
-    <x:row r="23" ht="48" customHeight="1">
+    <x:row r="23" ht="70.5" hidden="0" customHeight="1">
       <x:c r="A23" s="24" t="str">
-        <x:v>AUD-014</x:v>
+        <x:v>AUD-016</x:v>
       </x:c>
       <x:c r="B23" s="24" t="str">
-        <x:v>High</x:v>
+        <x:v>Medium</x:v>
       </x:c>
       <x:c r="C23" s="24" t="str">
-        <x:v>Implementation handoff</x:v>
+        <x:v>Approval</x:v>
       </x:c>
       <x:c r="D23" s="24" t="str">
-        <x:v>Issue a controlled SEED successor before integrated implementation verification.</x:v>
+        <x:v>Approve or return the narrow inspection amendment.</x:v>
       </x:c>
       <x:c r="E23" s="24" t="str">
-        <x:v>Requirements owner</x:v>
+        <x:v>Project Owner</x:v>
       </x:c>
       <x:c r="F23" s="24" t="str">
-        <x:v>One reproducible end-to-end test baseline</x:v>
+        <x:v>Bounded procurement-user release visibility</x:v>
       </x:c>
       <x:c r="G23" s="24" t="str">
         <x:v>Open</x:v>
       </x:c>
       <x:c r="H23" s="24" t="str">
-        <x:v>G1-REG-001 v1.1; SEED-001 v1.3 compared with current baseline</x:v>
+        <x:v>AUTH-ADR-001 v1.10 control block</x:v>
       </x:c>
       <x:c r="I23" s="2"/>
       <x:c r="J23" s="2"/>
@@ -2758,31 +2758,15 @@
       <x:c r="Y23" s="2"/>
       <x:c r="Z23" s="2"/>
     </x:row>
-    <x:row r="24" ht="48" customHeight="1">
-      <x:c r="A24" s="24" t="str">
-        <x:v>AUD-015</x:v>
-      </x:c>
-      <x:c r="B24" s="24" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="C24" s="24" t="str">
-        <x:v>Approval</x:v>
-      </x:c>
-      <x:c r="D24" s="24" t="str">
-        <x:v>Review and approve with STD-TPL-001 v0.10 before Claude Code implements the template runtime.</x:v>
-      </x:c>
-      <x:c r="E24" s="24" t="str">
-        <x:v>Project Owner</x:v>
-      </x:c>
-      <x:c r="F24" s="24" t="str">
-        <x:v>Authoritative STD runtime implementation</x:v>
-      </x:c>
-      <x:c r="G24" s="24" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="H24" s="24" t="str">
-        <x:v>STD-TPL-IMP-001 v1.0 control block</x:v>
-      </x:c>
+    <x:row r="24" ht="42" hidden="0" customHeight="1">
+      <x:c r="A24" s="24"/>
+      <x:c r="B24" s="24"/>
+      <x:c r="C24" s="24"/>
+      <x:c r="D24" s="24"/>
+      <x:c r="E24" s="24"/>
+      <x:c r="F24" s="24"/>
+      <x:c r="G24" s="24"/>
+      <x:c r="H24" s="24"/>
       <x:c r="I24" s="2"/>
       <x:c r="J24" s="2"/>
       <x:c r="K24" s="2"/>
@@ -2803,30 +2787,14 @@
       <x:c r="Z24" s="2"/>
     </x:row>
     <x:row r="25" ht="48" customHeight="1">
-      <x:c r="A25" s="24" t="str">
-        <x:v>AUD-016</x:v>
-      </x:c>
-      <x:c r="B25" s="24" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="C25" s="24" t="str">
-        <x:v>Approval</x:v>
-      </x:c>
-      <x:c r="D25" s="24" t="str">
-        <x:v>Approve or return the narrow inspection amendment.</x:v>
-      </x:c>
-      <x:c r="E25" s="24" t="str">
-        <x:v>Project Owner</x:v>
-      </x:c>
-      <x:c r="F25" s="24" t="str">
-        <x:v>Bounded procurement-user release visibility</x:v>
-      </x:c>
-      <x:c r="G25" s="24" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="H25" s="24" t="str">
-        <x:v>AUTH-ADR-001 v1.10 control block</x:v>
-      </x:c>
+      <x:c r="A25" s="24"/>
+      <x:c r="B25" s="24"/>
+      <x:c r="C25" s="24"/>
+      <x:c r="D25" s="24"/>
+      <x:c r="E25" s="24"/>
+      <x:c r="F25" s="24"/>
+      <x:c r="G25" s="24"/>
+      <x:c r="H25" s="24"/>
       <x:c r="I25" s="2"/>
       <x:c r="J25" s="2"/>
       <x:c r="K25" s="2"/>
@@ -8367,7 +8335,7 @@
         <x:v>Tenders</x:v>
       </x:c>
       <x:c r="C12" s="2" t="str">
-        <x:v>0.11</x:v>
+        <x:v>0.12</x:v>
       </x:c>
       <x:c r="D12" s="24" t="str">
         <x:v>Tender Preparation and Publication</x:v>
@@ -8376,11 +8344,13 @@
         <x:v>Module requirements</x:v>
       </x:c>
       <x:c r="F12" s="24" t="str">
-        <x:v>Project Owner review</x:v>
-      </x:c>
-      <x:c r="G12" s="36"/>
+        <x:v>Approved requirement</x:v>
+      </x:c>
+      <x:c r="G12" s="36" t="n">
+        <x:v>46291</x:v>
+      </x:c>
       <x:c r="H12" s="24" t="str">
-        <x:v>v0.10 on approval</x:v>
+        <x:v>v0.11 proposed, never approved</x:v>
       </x:c>
       <x:c r="I12" s="24" t="str">
         <x:v>Planned</x:v>
@@ -8392,19 +8362,19 @@
         <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="L12" s="2" t="str">
-        <x:v>Proposed</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="M12" s="24" t="str">
-        <x:v>Tender preparation, approval, publication, clarification, candidate notices, addenda and bound STD-release lifecycle.</x:v>
+        <x:v>Approved Tender preparation, approval, publication, clarifications, addenda, cancellation, bound STD-release lifecycle and KT-STD-001 v1.8 journey guidance.</x:v>
       </x:c>
       <x:c r="N12" s="24" t="str">
-        <x:v>REQ-CHG-001 v1.12; CFG-CHG-002 v0.16; STD-TPL-001 v0.10; STD-TPL-IMP-001 v1.0; BDS-CHG-001 v0.7</x:v>
+        <x:v>REQ-CHG-001 v1.12; CFG-CHG-002 v0.16; STD-TPL-001 v0.10; STD-TPL-IMP-001 v1.1; BDS-CHG-001 v0.7</x:v>
       </x:c>
       <x:c r="O12" s="24" t="str">
-        <x:v>Approve v0.11, then implement Available-only binding, Superseded continuation checks and Withdrawn blocking with no automatic rebinding.</x:v>
+        <x:v>Implement approved v0.12 and verify §§14–15; new binding requires an intact Available release switched On. Document approval is not production acceptance.</x:v>
       </x:c>
       <x:c r="P12" s="24" t="str">
-        <x:v>https://chatgpt.com/api/library/files/libfile_2709307394708191ad84161ab0c64d88/download</x:v>
+        <x:v>https://chatgpt.com/api/library/files/libfile_357a5c0bfd8881918423b65cb452bd41/download</x:v>
       </x:c>
       <x:c r="Q12" s="2"/>
       <x:c r="R12" s="2"/>
@@ -8422,10 +8392,10 @@
         <x:v>BDS-CHG-001</x:v>
       </x:c>
       <x:c r="B13" s="24" t="str">
-        <x:v>Supplier Workspace and Electronic Bid Submission</x:v>
+        <x:v>Supplier Portal and Electronic Bid Submission</x:v>
       </x:c>
       <x:c r="C13" s="2" t="str">
-        <x:v>0.7</x:v>
+        <x:v>0.8</x:v>
       </x:c>
       <x:c r="D13" s="24" t="str">
         <x:v>Supplier/Bidder Workspace and Bid Submission</x:v>
@@ -8434,11 +8404,13 @@
         <x:v>Module requirements</x:v>
       </x:c>
       <x:c r="F13" s="24" t="str">
-        <x:v>Project Owner review</x:v>
-      </x:c>
-      <x:c r="G13" s="36"/>
+        <x:v>Approved requirement</x:v>
+      </x:c>
+      <x:c r="G13" s="36" t="n">
+        <x:v>46291</x:v>
+      </x:c>
       <x:c r="H13" s="24" t="str">
-        <x:v>v0.6 on approval</x:v>
+        <x:v>v0.7 proposed, never approved; v0.6 and earlier historical</x:v>
       </x:c>
       <x:c r="I13" s="24" t="str">
         <x:v>Planned</x:v>
@@ -8450,19 +8422,19 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="L13" s="2" t="str">
-        <x:v>Proposed</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="M13" s="24" t="str">
-        <x:v>Public discovery, supplier access, metadata-driven bid preparation and atomic sealed submission handoff.</x:v>
+        <x:v>Public discovery, supplier Account, structured Goods/IT bid preparation, signature, receipt, replacement and sealed Bid Opening handoff, with actor-specific guidance and bound STD-release controls.</x:v>
       </x:c>
       <x:c r="N13" s="24" t="str">
-        <x:v>TPR-CHG-001; STD-TPL-001; CFG-CHG-002; AUTH-ADR-001</x:v>
+        <x:v>TPR-CHG-001 v0.12; STD-TPL-001 v0.10; STD-TPL-IMP-001 v1.1; CFG-CHG-002 v0.16; AUTH-ADR-001 v1.10; KT-STD-001 v1.8; G1-REG-001 v1.1</x:v>
       </x:c>
       <x:c r="O13" s="24" t="str">
-        <x:v>Approve requirements; keep production submission disabled until the operating profile and release gates pass.</x:v>
+        <x:v>Implement approved v0.8; keep production submission disabled until §§5.10 and 15 gates pass. Published-Tender Superseded/Withdrawn behavior remains conditional on approval of TPR-CHG-001 v0.13. Reconcile its §10 presentation with the newly approved KT-STD-001 v1.9 before design execution.</x:v>
       </x:c>
       <x:c r="P13" s="24" t="str">
-        <x:v>https://chatgpt.com/api/library/files/libfile_6a8aca132b408191a8d23c467408ecf4/download</x:v>
+        <x:v>https://chatgpt.com/api/library/files/libfile_7252e90793e4819199bca1d68fab4457/download</x:v>
       </x:c>
       <x:c r="Q13" s="2"/>
       <x:c r="R13" s="2"/>
@@ -8492,11 +8464,13 @@
         <x:v>Template standard</x:v>
       </x:c>
       <x:c r="F14" s="24" t="str">
-        <x:v>Project Owner review</x:v>
-      </x:c>
-      <x:c r="G14" s="36"/>
+        <x:v>Approved requirement</x:v>
+      </x:c>
+      <x:c r="G14" s="36" t="n">
+        <x:v>46291</x:v>
+      </x:c>
       <x:c r="H14" s="24" t="str">
-        <x:v>v0.9 on approval</x:v>
+        <x:v>v0.9 and earlier</x:v>
       </x:c>
       <x:c r="I14" s="24" t="str">
         <x:v>Planned</x:v>
@@ -8508,16 +8482,16 @@
         <x:v>Candidate</x:v>
       </x:c>
       <x:c r="L14" s="2" t="str">
-        <x:v>Proposed</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="M14" s="24" t="str">
-        <x:v>Controlled curation, structured gates, release comparison, administrative inspection, concern capture, shared compiler, renderer abstraction and exact release lifecycle.</x:v>
+        <x:v>Controlled template content and construction, installed integrity, administrative inspection and Administrator On/Off switch for new Tender binding.</x:v>
       </x:c>
       <x:c r="N14" s="24" t="str">
-        <x:v>KT-STD-001 v1.8; REQ-CHG-001 v1.12; TPR-CHG-001 v0.11; STD-TPL-IMP-001 v1.0; BDS-CHG-001 v0.7; CFG-CHG-002 v0.16</x:v>
+        <x:v>KT-STD-001 v1.8; REQ-CHG-001 v1.12; TPR-CHG-001 v0.12; STD-TPL-IMP-001 v1.1 approved; BDS-CHG-001 v0.7; CFG-CHG-002 v0.16</x:v>
       </x:c>
       <x:c r="O14" s="24" t="str">
-        <x:v>Approve v0.10, complete every release asset and gate, rebuild the exact candidate and obtain manifest-level owner approval.</x:v>
+        <x:v>Finish and verify release 1.1 assets; install the compatible digest-matched bundle On by default or Off by deployment request. No separate manifest approval.</x:v>
       </x:c>
       <x:c r="P14" s="24" t="str">
         <x:v>https://chatgpt.com/api/library/files/libfile_9a03e6ea43d88191938445a1a04d99b1/download</x:v>
@@ -8541,7 +8515,7 @@
         <x:v>Installed STD Template Runtime</x:v>
       </x:c>
       <x:c r="C15" s="2" t="str">
-        <x:v>1.0</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="D15" s="24" t="str">
         <x:v>STD Templates</x:v>
@@ -8550,11 +8524,13 @@
         <x:v>Implementation authority</x:v>
       </x:c>
       <x:c r="F15" s="24" t="str">
-        <x:v>Project Owner review</x:v>
-      </x:c>
-      <x:c r="G15" s="36"/>
+        <x:v>Approved requirement</x:v>
+      </x:c>
+      <x:c r="G15" s="36" t="n">
+        <x:v>46291</x:v>
+      </x:c>
       <x:c r="H15" s="24" t="str">
-        <x:v>v0.2 historical pack on approval</x:v>
+        <x:v>v1.0 proposed but never approved; v0.2 historical</x:v>
       </x:c>
       <x:c r="I15" s="24" t="str">
         <x:v>Planned</x:v>
@@ -8566,19 +8542,19 @@
         <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="L15" s="2" t="str">
-        <x:v>Proposed</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="M15" s="24" t="str">
-        <x:v>Immutable installed-release registry and assets, fail-closed installer, shared compiler, renderer adapters, inspection projections, concerns and lifecycle enforcement.</x:v>
+        <x:v>Immutable installed-release runtime, verified installation, shared compiler, renderer adapters, inspection and deployment-only per-site On/Off switch.</x:v>
       </x:c>
       <x:c r="N15" s="24" t="str">
-        <x:v>STD-TPL-001 v0.10; TPR-CHG-001 v0.11; BDS-CHG-001 v0.7; AUTH-ADR-001 v1.10; KT-STD-001 v1.8</x:v>
+        <x:v>STD-TPL-001 v0.10; TPR-CHG-001 v0.12; BDS-CHG-001 v0.7; AUTH-ADR-001 v1.10; KT-STD-001 v1.8</x:v>
       </x:c>
       <x:c r="O15" s="24" t="str">
-        <x:v>Approve as the implementation authority and implement before relying on release 1.1 in Tenders or Bid Submission.</x:v>
+        <x:v>Implement approved v1.1; reconcile TPR, REQ, BDS and Gate 1 references to OD5. The bundle remains uninstalled and unverified.</x:v>
       </x:c>
       <x:c r="P15" s="24" t="str">
-        <x:v>https://chatgpt.com/api/library/files/libfile_686f793d1d8c8191a192135f10ea74e8/download</x:v>
+        <x:v>https://chatgpt.com/api/library/files/libfile_87bca073b1b081918cc5cefdff08adcc/download</x:v>
       </x:c>
       <x:c r="Q15" s="2"/>
       <x:c r="R15" s="2"/>
@@ -8599,7 +8575,7 @@
         <x:v>Document, Design and Verification Standards</x:v>
       </x:c>
       <x:c r="C16" s="2" t="str">
-        <x:v>1.8</x:v>
+        <x:v>1.9</x:v>
       </x:c>
       <x:c r="D16" s="24" t="str">
         <x:v>All</x:v>
@@ -8611,10 +8587,10 @@
         <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="G16" s="36" t="n">
-        <x:v>46290</x:v>
+        <x:v>46291</x:v>
       </x:c>
       <x:c r="H16" s="24" t="str">
-        <x:v>v1.7 approved 21 September 2026; v1.6 and earlier remain historical evidence</x:v>
+        <x:v>v1.8 approved 25 September 2026; v1.7 and earlier remain historical evidence</x:v>
       </x:c>
       <x:c r="I16" s="24" t="str">
         <x:v>Not applicable</x:v>
@@ -8629,16 +8605,16 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="M16" s="24" t="str">
-        <x:v>Current cross-cutting design and verification authority. Adds the restrained next-step block and journey tracker, server-produced next-step contract, guard reasons, hand-off register, My Work, Home and dead-end conformance test to the v1.7 baseline.</x:v>
+        <x:v>Current cross-cutting design and verification authority. Refines the white page sheet, guidance-region placement and restrained accent rules; retains the v1.8 next-step, journey, guard-reason, hand-off, My Work, Home and dead-end conformance contracts.</x:v>
       </x:c>
       <x:c r="N16" s="24" t="str">
         <x:v>Workflow Guidance Standard; all controlled change documents</x:v>
       </x:c>
       <x:c r="O16" s="24" t="str">
-        <x:v>Apply v1.8 to every new or revised change unit, artboard prompt, implementation contract and release verification.</x:v>
+        <x:v>Apply v1.9 to every new or revised change unit and artboard prompt; retain the v1.8 runtime and verification contracts carried forward into v1.9.</x:v>
       </x:c>
       <x:c r="P16" s="24" t="str">
-        <x:v>https://chatgpt.com/api/library/files/libfile_ed139679ea5c8191bda6f73eed748929/download</x:v>
+        <x:v>https://chatgpt.com/api/library/files/libfile_c189a864c48c81918002bab99a3dc04c/download</x:v>
       </x:c>
       <x:c r="Q16" s="2"/>
       <x:c r="R16" s="2"/>
@@ -9034,16 +9010,16 @@
         <x:v>Not applicable</x:v>
       </x:c>
       <x:c r="L23" s="2" t="str">
-        <x:v>Yes—through KT-STD-001 v1.8 and module adoption</x:v>
+        <x:v>Yes—through KT-STD-001 v1.9 and module adoption</x:v>
       </x:c>
       <x:c r="M23" s="24" t="str">
         <x:v>Defines the no-dead-ends test, shared next-step response, My Work hand-off coverage, restrained journey tracker and Home guidance using the Planning over-budget case.</x:v>
       </x:c>
       <x:c r="N23" s="24" t="str">
-        <x:v>KT-STD-001 v1.8; module-specific adoption</x:v>
+        <x:v>KT-STD-001 v1.9; module-specific adoption</x:v>
       </x:c>
       <x:c r="O23" s="24" t="str">
-        <x:v>Retain as approved provenance. Implement operative wording from KT-STD-001 v1.8 and each current module document.</x:v>
+        <x:v>Retain as approved provenance. Implement operative wording from KT-STD-001 v1.9 and each current module document.</x:v>
       </x:c>
       <x:c r="P23" s="24" t="str">
         <x:v>https://chatgpt.com/api/library/files/libfile_ac20011f049881919843681b0461c5cb/download</x:v>
@@ -9263,13 +9239,13 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="M27" s="24" t="str">
-        <x:v>Existing generated renderer/review-pack artefacts; candidate must be reconciled to STD-TPL-001 v0.10 and installed under STD-TPL-IMP-001 v1.0 before use.</x:v>
+        <x:v>Earlier candidate ZIP; requires reconciliation to amended STD-TPL-001 v0.10 before installation and Administrator On.</x:v>
       </x:c>
       <x:c r="N27" s="24" t="str">
-        <x:v>STD-TPL-001 v0.10; STD-TPL-IMP-001 v1.0</x:v>
+        <x:v>STD-TPL-001 v0.10; STD-TPL-IMP-001 v1.1</x:v>
       </x:c>
       <x:c r="O27" s="24" t="str">
-        <x:v>Rebuild and verify structured gates, change report, exact manifest, compiler vectors and renderer adapter; do not treat the existing ZIP as an approved release.</x:v>
+        <x:v>Rebuild and verify the bundle and renderer compatibility; do not treat this earlier ZIP as installed or On.</x:v>
       </x:c>
       <x:c r="P27" s="24" t="str">
         <x:v>https://chatgpt.com/api/library/files/libfile_7350870ee594819189729148528d97d7/download</x:v>
@@ -14234,7 +14210,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42318d86bf824067"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71655390f1ff431c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14626,7 +14602,7 @@
         <x:v>Not evidenced</x:v>
       </x:c>
       <x:c r="H10" s="24" t="str">
-        <x:v>REQ-CHG-001 v1.12 / TPR-CHG-001 v0.11</x:v>
+        <x:v>REQ-CHG-001 v1.12 / TPR-CHG-001 v0.12</x:v>
       </x:c>
       <x:c r="I10" s="24" t="str">
         <x:v>Tender creation must reject missing, stale or unauthorised handoff data.</x:v>
@@ -14706,10 +14682,10 @@
         <x:v>Requisitions/Tenders/Bids</x:v>
       </x:c>
       <x:c r="D12" s="24" t="str">
-        <x:v>Exact approved release manifest, structured gates, change report, shared compiler, renderer adapter and lifecycle</x:v>
+        <x:v>Digest-matched installed template, construction evidence, shared compiler, renderer adapter and site On/Off switch</x:v>
       </x:c>
       <x:c r="E12" s="24" t="str">
-        <x:v>Needs approval and rebuild</x:v>
+        <x:v>STD v0.10 and runtime v1.1 approved; bundle pending</x:v>
       </x:c>
       <x:c r="F12" s="24" t="str">
         <x:v>Planned</x:v>
@@ -14718,10 +14694,10 @@
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="H12" s="24" t="str">
-        <x:v>STD-TPL-001 v0.10 / STD-TPL-IMP-001 v1.0</x:v>
+        <x:v>STD-TPL-001 v0.10 / STD-TPL-IMP-001 v1.1</x:v>
       </x:c>
       <x:c r="I12" s="24" t="str">
-        <x:v>No module may infer missing semantics, use an unapproved manifest, duplicate the compiler or bypass release lifecycle.</x:v>
+        <x:v>No module may infer missing semantics, bypass integrity/renderer checks, or bind a new Tender while the site switch is Off.</x:v>
       </x:c>
       <x:c r="J12" s="2"/>
       <x:c r="K12" s="2"/>
@@ -14764,7 +14740,7 @@
         <x:v>Not evidenced</x:v>
       </x:c>
       <x:c r="H13" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.11 / BDS-CHG-001 v0.7 / STD-TPL-IMP-001 v1.0</x:v>
+        <x:v>TPR-CHG-001 v0.12 / BDS-CHG-001 v0.8 / STD-TPL-IMP-001 v1.1</x:v>
       </x:c>
       <x:c r="I13" s="24" t="str">
         <x:v>Bid UI must be generated only by the shared compiler from the exact effective published definition and release identity.</x:v>
@@ -14810,7 +14786,7 @@
         <x:v>Not evidenced</x:v>
       </x:c>
       <x:c r="H14" s="24" t="str">
-        <x:v>BDS-CHG-001 v0.7 / TPR-CHG-001 v0.11</x:v>
+        <x:v>BDS-CHG-001 v0.8 / TPR-CHG-001 v0.12</x:v>
       </x:c>
       <x:c r="I14" s="24" t="str">
         <x:v>Start bid must not create a half-registered candidate or orphan question.</x:v>
@@ -14948,7 +14924,7 @@
         <x:v>Not evidenced</x:v>
       </x:c>
       <x:c r="H17" s="24" t="str">
-        <x:v>KT-STD-001 v1.8 / current module document</x:v>
+        <x:v>KT-STD-001 v1.9 / current module document</x:v>
       </x:c>
       <x:c r="I17" s="24" t="str">
         <x:v>No authorised user may reach a meaningful record state without an action, waiting owner, correctable blocker or completed outcome.</x:v>
@@ -14994,7 +14970,7 @@
         <x:v>Not evidenced</x:v>
       </x:c>
       <x:c r="H18" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.11 / BDS-CHG-001 v0.7</x:v>
+        <x:v>TPR-CHG-001 v0.12 / BDS-CHG-001 v0.8</x:v>
       </x:c>
       <x:c r="I18" s="24" t="str">
         <x:v>Changed requirements require an issued addendum; clarifications alone cannot mutate the bid definition.</x:v>
@@ -15028,7 +15004,7 @@
         <x:v>Tenders/Bid Submission</x:v>
       </x:c>
       <x:c r="D19" s="24" t="str">
-        <x:v>Bound release lifecycle projection</x:v>
+        <x:v>Bound release and site availability projection</x:v>
       </x:c>
       <x:c r="E19" s="24" t="str">
         <x:v>Closed in requirements</x:v>
@@ -15040,10 +15016,10 @@
         <x:v>Not evidenced</x:v>
       </x:c>
       <x:c r="H19" s="24" t="str">
-        <x:v>STD-TPL-001 v0.10 / STD-TPL-IMP-001 v1.0 / TPR-CHG-001 v0.11</x:v>
+        <x:v>STD-TPL-001 v0.10 / STD-TPL-IMP-001 v1.1 / TPR-CHG-001 v0.12</x:v>
       </x:c>
       <x:c r="I19" s="24" t="str">
-        <x:v>New binding requires Available; Superseded continuation requires integrity; Withdrawn blocks unpublished continuation; no automatic rebind.</x:v>
+        <x:v>New binding requires site On and valid integrity/renderer; Off preserves existing bindings, safety/legal withdrawal blocks affected unpublished publication; never automatically rebind.</x:v>
       </x:c>
       <x:c r="J19" s="2"/>
       <x:c r="K19" s="2"/>
@@ -15086,7 +15062,7 @@
         <x:v>Not started</x:v>
       </x:c>
       <x:c r="H20" s="24" t="str">
-        <x:v>BDS-CHG-001 v0.7</x:v>
+        <x:v>BDS-CHG-001 v0.8</x:v>
       </x:c>
       <x:c r="I20" s="24" t="str">
         <x:v>Gate 1 ends at sealed handoff; no opening or evaluation behaviour is implied.</x:v>
@@ -20189,7 +20165,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4755ccc4c084e74"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02c7118153cc4ed9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20502,7 +20478,7 @@
         <x:v>Release tooling is controlled and manifest-based.</x:v>
       </x:c>
       <x:c r="F9" s="24" t="str">
-        <x:v>Admin UI is inspection and approval status, not raw schema editing.</x:v>
+        <x:v>Admin UI shows content and site On/Off state, never a generic schema editor.</x:v>
       </x:c>
       <x:c r="G9" s="2"/>
       <x:c r="H9" s="2"/>
@@ -21016,7 +20992,7 @@
         <x:v>Approved</x:v>
       </x:c>
       <x:c r="D22" s="24" t="str">
-        <x:v>KT-STD-001 v1.8 / current module document</x:v>
+        <x:v>KT-STD-001 v1.9 / current module document</x:v>
       </x:c>
       <x:c r="E22" s="24" t="str">
         <x:v>Centralise next-step and guard evaluation and test every supported persona/state pair.</x:v>
@@ -21136,7 +21112,7 @@
         <x:v>Approved</x:v>
       </x:c>
       <x:c r="D25" s="24" t="str">
-        <x:v>KT-STD-001 v1.8 / Workflow Guidance Standard</x:v>
+        <x:v>KT-STD-001 v1.9 / Workflow Guidance Standard</x:v>
       </x:c>
       <x:c r="E25" s="24" t="str">
         <x:v>Derive restrained journey context from authoritative workflow state and hand-offs.</x:v>
@@ -21170,19 +21146,19 @@
         <x:v>DEC-021</x:v>
       </x:c>
       <x:c r="B26" s="24" t="str">
-        <x:v>STD Templates is a transparent inspection and concern surface, not a runtime legal-template editor or second site-approval workflow.</x:v>
+        <x:v>STD Templates provides inspection and concern capture; an audited deployment-only command switches template use On or Off.</x:v>
       </x:c>
       <x:c r="C26" s="2" t="str">
-        <x:v>Proposed</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="D26" s="24" t="str">
-        <x:v>STD-TPL-001 v0.10 / STD-TPL-IMP-001 v1.0</x:v>
+        <x:v>STD-TPL-001 v0.10 / FU-01 OD5</x:v>
       </x:c>
       <x:c r="E26" s="24" t="str">
-        <x:v>Install exact approved assets and expose projections; prohibit editable content DocTypes.</x:v>
+        <x:v>Install verified immutable assets On by default or Off on request; prohibit editable content DocTypes and Desk switching.</x:v>
       </x:c>
       <x:c r="F26" s="24" t="str">
-        <x:v>Show coverage, exclusions, changes and gates with bounded Report concern.</x:v>
+        <x:v>Show coverage and switch state; no Desk switch.</x:v>
       </x:c>
       <x:c r="G26" s="2"/>
       <x:c r="H26" s="2"/>
@@ -21213,10 +21189,10 @@
         <x:v>Fixture and production Bid-definition generation use one deterministic compiler and releases bind a versioned renderer adapter.</x:v>
       </x:c>
       <x:c r="C27" s="2" t="str">
-        <x:v>Proposed</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="D27" s="24" t="str">
-        <x:v>STD-TPL-001 v0.10 / STD-TPL-IMP-001 v1.0</x:v>
+        <x:v>STD-TPL-001 v0.10 / STD-TPL-IMP-001 v1.1</x:v>
       </x:c>
       <x:c r="E27" s="24" t="str">
         <x:v>One compiler implementation; adapter-bound rendering; no arbitrary fallback.</x:v>
@@ -21250,19 +21226,19 @@
         <x:v>DEC-023</x:v>
       </x:c>
       <x:c r="B28" s="24" t="str">
-        <x:v>A release lifecycle change never automatically rebinds a Tender; Superseded may continue only with integrity, while Withdrawn blocks unpublished continuation.</x:v>
+        <x:v>Turning a release Off does not automatically rebind or block an already-bound Tender; safety/legal withdrawal blocks affected unpublished publication.</x:v>
       </x:c>
       <x:c r="C28" s="2" t="str">
-        <x:v>Proposed</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="D28" s="24" t="str">
-        <x:v>STD-TPL-001 v0.10 / TPR-CHG-001 v0.11</x:v>
+        <x:v>STD-TPL-001 v0.10 / TPR-CHG-001 v0.12</x:v>
       </x:c>
       <x:c r="E28" s="24" t="str">
-        <x:v>Enforce the action matrix at every boundary and preserve published history.</x:v>
+        <x:v>Preserve exact bindings and published history; apply the specific withdrawal exception.</x:v>
       </x:c>
       <x:c r="F28" s="24" t="str">
-        <x:v>Show successor/withdrawal notice and one governed next step without an upgrade selector.</x:v>
+        <x:v>Show the site switch consequence and any withdrawal reason.</x:v>
       </x:c>
       <x:c r="G28" s="2"/>
       <x:c r="H28" s="2"/>
@@ -21285,13 +21261,25 @@
       <x:c r="Y28" s="2"/>
       <x:c r="Z28" s="2"/>
     </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="2"/>
-      <x:c r="B29" s="2"/>
-      <x:c r="C29" s="2"/>
-      <x:c r="D29" s="2"/>
-      <x:c r="E29" s="2"/>
-      <x:c r="F29" s="2"/>
+    <x:row r="29" ht="63" customHeight="1">
+      <x:c r="A29" s="24" t="str">
+        <x:v>DEC-024</x:v>
+      </x:c>
+      <x:c r="B29" s="24" t="str">
+        <x:v>Template use for new Tenders is a deployment-only per-site On/Off switch; installation needs no owner approval and sets On by default unless Off is requested.</x:v>
+      </x:c>
+      <x:c r="C29" s="24" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="D29" s="24" t="str">
+        <x:v>STD-TPL-001 v0.10 / FU-01 OD5, 2026-09-26</x:v>
+      </x:c>
+      <x:c r="E29" s="24" t="str">
+        <x:v>New binding requires exactly one On Available release per template key; multiple On releases refuse binding. Existing bindings stay pinned.</x:v>
+      </x:c>
+      <x:c r="F29" s="24" t="str">
+        <x:v>Read-only On/Off state in STD Templates, with actor and time.</x:v>
+      </x:c>
       <x:c r="G29" s="2"/>
       <x:c r="H29" s="2"/>
       <x:c r="I29" s="2"/>
@@ -26119,7 +26107,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4db4c67d08734802"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09de1e094824414d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26378,7 +26366,7 @@
         <x:v>CFG-CHG-002 v0.16 / STD-TPL-001 v0.10</x:v>
       </x:c>
       <x:c r="G7" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Mixed approved/proposed</x:v>
       </x:c>
       <x:c r="H7" s="24" t="str">
         <x:v>Yes</x:v>
@@ -26426,7 +26414,7 @@
         <x:v>STD-TPL-001 v0.10</x:v>
       </x:c>
       <x:c r="G8" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H8" s="24" t="str">
         <x:v>Yes</x:v>
@@ -26474,7 +26462,7 @@
         <x:v>STD-TPL-001 v0.10</x:v>
       </x:c>
       <x:c r="G9" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H9" s="24" t="str">
         <x:v>Yes</x:v>
@@ -26510,19 +26498,19 @@
         <x:v>STD Templates</x:v>
       </x:c>
       <x:c r="C10" s="24" t="str">
-        <x:v>Verify and approve the exact release manifest.</x:v>
+        <x:v>Verify the installed release and provide a deployment-only site On/Off switch.</x:v>
       </x:c>
       <x:c r="D10" s="24" t="str">
-        <x:v>Digest-bound owner approval of the rebuilt bundle.</x:v>
+        <x:v>Check manifest and assets during installation; install On by default or Off by deployment request.</x:v>
       </x:c>
       <x:c r="E10" s="24" t="str">
-        <x:v>Exact blocker and approval identity visible.</x:v>
+        <x:v>Show the read-only switch state and specific integrity/compatibility errors.</x:v>
       </x:c>
       <x:c r="F10" s="24" t="str">
         <x:v>STD-TPL-001 v0.10</x:v>
       </x:c>
       <x:c r="G10" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H10" s="24" t="str">
         <x:v>Yes</x:v>
@@ -26567,10 +26555,10 @@
         <x:v>Name the source problem and owner without technical codes.</x:v>
       </x:c>
       <x:c r="F11" s="24" t="str">
-        <x:v>REQ-CHG-001 v1.12 / TPR-CHG-001 v0.11</x:v>
+        <x:v>REQ-CHG-001 v1.12 / TPR-CHG-001 v0.12</x:v>
       </x:c>
       <x:c r="G11" s="24" t="str">
-        <x:v>Mixed approved/proposed</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H11" s="24" t="str">
         <x:v>Yes</x:v>
@@ -26606,19 +26594,19 @@
         <x:v>Tenders</x:v>
       </x:c>
       <x:c r="C12" s="24" t="str">
-        <x:v>Prepare tender from exact approved template release.</x:v>
+        <x:v>Prepare Tender from an exact installed template that is On for new binding.</x:v>
       </x:c>
       <x:c r="D12" s="24" t="str">
-        <x:v>Bind template, renderer and response schema identities.</x:v>
+        <x:v>Bind template, renderer and response schema identities only when exactly one release is On and checks pass.</x:v>
       </x:c>
       <x:c r="E12" s="24" t="str">
         <x:v>Progressive preparation journey with concise supporting detail.</x:v>
       </x:c>
       <x:c r="F12" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.11 / STD-TPL-001 v0.10</x:v>
+        <x:v>TPR-CHG-001 v0.12 / STD-TPL-001 v0.10</x:v>
       </x:c>
       <x:c r="G12" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H12" s="24" t="str">
         <x:v>Yes</x:v>
@@ -26663,10 +26651,10 @@
         <x:v>Clear confirmed/evidence-required states and direct actions.</x:v>
       </x:c>
       <x:c r="F13" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.11</x:v>
+        <x:v>TPR-CHG-001 v0.12</x:v>
       </x:c>
       <x:c r="G13" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H13" s="24" t="str">
         <x:v>Yes</x:v>
@@ -26711,10 +26699,10 @@
         <x:v>One understandable clarification feed.</x:v>
       </x:c>
       <x:c r="F14" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.11 / BDS-CHG-001 v0.7</x:v>
+        <x:v>TPR-CHG-001 v0.12 / BDS-CHG-001 v0.8</x:v>
       </x:c>
       <x:c r="G14" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H14" s="24" t="str">
         <x:v>No</x:v>
@@ -26759,10 +26747,10 @@
         <x:v>Prominent change notice and acknowledgement state.</x:v>
       </x:c>
       <x:c r="F15" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.11 / BDS-CHG-001 v0.7</x:v>
+        <x:v>TPR-CHG-001 v0.12 / BDS-CHG-001 v0.8</x:v>
       </x:c>
       <x:c r="G15" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H15" s="24" t="str">
         <x:v>Yes</x:v>
@@ -26807,10 +26795,10 @@
         <x:v>Simple search/list/detail; reusable framework pages where suitable.</x:v>
       </x:c>
       <x:c r="F16" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.11 / BDS-CHG-001 v0.7</x:v>
+        <x:v>TPR-CHG-001 v0.12 / BDS-CHG-001 v0.8</x:v>
       </x:c>
       <x:c r="G16" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H16" s="24" t="str">
         <x:v>Yes</x:v>
@@ -26855,10 +26843,10 @@
         <x:v>Direct access with minimal account friction.</x:v>
       </x:c>
       <x:c r="F17" s="24" t="str">
-        <x:v>BDS-CHG-001 v0.7</x:v>
+        <x:v>BDS-CHG-001 v0.8</x:v>
       </x:c>
       <x:c r="G17" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H17" s="24" t="str">
         <x:v>Yes</x:v>
@@ -26903,10 +26891,10 @@
         <x:v>Never expose cross-supplier records or selectors.</x:v>
       </x:c>
       <x:c r="F18" s="24" t="str">
-        <x:v>BDS-CHG-001 v0.7 / AUTH-ADR-001 v1.10</x:v>
+        <x:v>BDS-CHG-001 v0.8 / AUTH-ADR-001 v1.10</x:v>
       </x:c>
       <x:c r="G18" s="24" t="str">
-        <x:v>Mixed proposed/approved</x:v>
+        <x:v>Mixed approved/proposed</x:v>
       </x:c>
       <x:c r="H18" s="24" t="str">
         <x:v>Yes</x:v>
@@ -26951,10 +26939,10 @@
         <x:v>Single Start bid action and deterministic recovery.</x:v>
       </x:c>
       <x:c r="F19" s="24" t="str">
-        <x:v>BDS-CHG-001 v0.7</x:v>
+        <x:v>BDS-CHG-001 v0.8</x:v>
       </x:c>
       <x:c r="G19" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H19" s="24" t="str">
         <x:v>Yes</x:v>
@@ -26999,10 +26987,10 @@
         <x:v>Goods, Works and Services differ through metadata, not bespoke page forks.</x:v>
       </x:c>
       <x:c r="F20" s="24" t="str">
-        <x:v>BDS-CHG-001 v0.7 / STD-TPL-001 v0.10</x:v>
+        <x:v>BDS-CHG-001 v0.8 / STD-TPL-001 v0.10</x:v>
       </x:c>
       <x:c r="G20" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H20" s="24" t="str">
         <x:v>Yes</x:v>
@@ -27047,10 +27035,10 @@
         <x:v>Short, structured task sections with progress and actionable errors.</x:v>
       </x:c>
       <x:c r="F21" s="24" t="str">
-        <x:v>BDS-CHG-001 v0.7</x:v>
+        <x:v>BDS-CHG-001 v0.8</x:v>
       </x:c>
       <x:c r="G21" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H21" s="24" t="str">
         <x:v>Yes</x:v>
@@ -27095,10 +27083,10 @@
         <x:v>Explain exactly what changed and what the supplier must revisit.</x:v>
       </x:c>
       <x:c r="F22" s="24" t="str">
-        <x:v>BDS-CHG-001 v0.7</x:v>
+        <x:v>BDS-CHG-001 v0.8</x:v>
       </x:c>
       <x:c r="G22" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H22" s="24" t="str">
         <x:v>Yes</x:v>
@@ -27143,10 +27131,10 @@
         <x:v>Approved temporary-unavailability message; drafts remain safe.</x:v>
       </x:c>
       <x:c r="F23" s="24" t="str">
-        <x:v>BDS-CHG-001 v0.7 / CFG-CHG-002 v0.16</x:v>
+        <x:v>BDS-CHG-001 v0.8 / CFG-CHG-002 v0.16</x:v>
       </x:c>
       <x:c r="G23" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Mixed approved/proposed</x:v>
       </x:c>
       <x:c r="H23" s="24" t="str">
         <x:v>Yes</x:v>
@@ -27191,10 +27179,10 @@
         <x:v>Plain explanation of authority and consequence.</x:v>
       </x:c>
       <x:c r="F24" s="24" t="str">
-        <x:v>BDS-CHG-001 v0.7 / STD-TPL-001 v0.10</x:v>
+        <x:v>BDS-CHG-001 v0.8 / STD-TPL-001 v0.10</x:v>
       </x:c>
       <x:c r="G24" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H24" s="24" t="str">
         <x:v>Yes</x:v>
@@ -27239,10 +27227,10 @@
         <x:v>Show only the instrument actually required.</x:v>
       </x:c>
       <x:c r="F25" s="24" t="str">
-        <x:v>BDS-CHG-001 v0.7 / STD-TPL-001 v0.10</x:v>
+        <x:v>BDS-CHG-001 v0.8 / STD-TPL-001 v0.10</x:v>
       </x:c>
       <x:c r="G25" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H25" s="24" t="str">
         <x:v>Yes</x:v>
@@ -27287,10 +27275,10 @@
         <x:v>Clear submitted state and downloadable receipt.</x:v>
       </x:c>
       <x:c r="F26" s="24" t="str">
-        <x:v>BDS-CHG-001 v0.7</x:v>
+        <x:v>BDS-CHG-001 v0.8</x:v>
       </x:c>
       <x:c r="G26" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H26" s="24" t="str">
         <x:v>Yes</x:v>
@@ -27431,10 +27419,10 @@
         <x:v>No hidden or partial enablement.</x:v>
       </x:c>
       <x:c r="F29" s="24" t="str">
-        <x:v>G1-REG-001 v1.1 / BDS-CHG-001 v0.7</x:v>
+        <x:v>G1-REG-001 v1.1 / BDS-CHG-001 v0.8</x:v>
       </x:c>
       <x:c r="G29" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H29" s="24" t="str">
         <x:v>Yes</x:v>
@@ -27473,16 +27461,16 @@
         <x:v>Implement the exact installed-release runtime authority.</x:v>
       </x:c>
       <x:c r="D30" s="24" t="str">
-        <x:v>Immutable registry/assets, transactionally verified installation and owner projections.</x:v>
+        <x:v>Immutable registry/assets, verified installation and audited deployment-only On/Off switch.</x:v>
       </x:c>
       <x:c r="E30" s="24" t="str">
-        <x:v>No new authoring or adoption-approval surface.</x:v>
+        <x:v>Read-only state in STD Templates; no template editing or adoption approval.</x:v>
       </x:c>
       <x:c r="F30" s="24" t="str">
-        <x:v>STD-TPL-IMP-001 v1.0</x:v>
+        <x:v>STD-TPL-IMP-001 v1.1</x:v>
       </x:c>
       <x:c r="G30" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H30" s="24" t="str">
         <x:v>Yes</x:v>
@@ -27527,10 +27515,10 @@
         <x:v>Coverage and changes section with plain summaries and drill-down, not raw JSON.</x:v>
       </x:c>
       <x:c r="F31" s="24" t="str">
-        <x:v>STD-TPL-001 v0.10 / STD-TPL-IMP-001 v1.0</x:v>
+        <x:v>STD-TPL-001 v0.10 / STD-TPL-IMP-001 v1.1</x:v>
       </x:c>
       <x:c r="G31" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Mixed approved/proposed</x:v>
       </x:c>
       <x:c r="H31" s="24" t="str">
         <x:v>Yes</x:v>
@@ -27578,7 +27566,7 @@
         <x:v>STD-TPL-001 v0.10 / AUTH-ADR-001 v1.10</x:v>
       </x:c>
       <x:c r="G32" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Mixed approved/proposed</x:v>
       </x:c>
       <x:c r="H32" s="24" t="str">
         <x:v>No</x:v>
@@ -27623,10 +27611,10 @@
         <x:v>Technical identities remain collapsed; routine failure copy is direct.</x:v>
       </x:c>
       <x:c r="F33" s="24" t="str">
-        <x:v>STD-TPL-001 v0.10 / STD-TPL-IMP-001 v1.0</x:v>
+        <x:v>STD-TPL-001 v0.10 / STD-TPL-IMP-001 v1.1</x:v>
       </x:c>
       <x:c r="G33" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Mixed approved/proposed</x:v>
       </x:c>
       <x:c r="H33" s="24" t="str">
         <x:v>Yes</x:v>
@@ -27671,10 +27659,10 @@
         <x:v>Show successor notice and preserved exact release.</x:v>
       </x:c>
       <x:c r="F34" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.11 / STD-TPL-001 v0.10</x:v>
+        <x:v>TPR-CHG-001 v0.12 / STD-TPL-001 v0.10</x:v>
       </x:c>
       <x:c r="G34" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H34" s="24" t="str">
         <x:v>Yes</x:v>
@@ -27719,10 +27707,10 @@
         <x:v>Direct reason, release link and governed next step.</x:v>
       </x:c>
       <x:c r="F35" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.11 / STD-TPL-001 v0.10</x:v>
+        <x:v>TPR-CHG-001 v0.12 / STD-TPL-001 v0.10</x:v>
       </x:c>
       <x:c r="G35" s="24" t="str">
-        <x:v>Project Owner review</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H35" s="24" t="str">
         <x:v>Yes</x:v>
@@ -27911,10 +27899,10 @@
         <x:v>Show concise confirmed treatment with correction route.</x:v>
       </x:c>
       <x:c r="F39" s="24" t="str">
-        <x:v>REQ-CHG-001 v1.12 / TPR-CHG-001 v0.11 / BDS-CHG-001 v0.7</x:v>
+        <x:v>REQ-CHG-001 v1.12 / TPR-CHG-001 v0.12 / BDS-CHG-001 v0.8</x:v>
       </x:c>
       <x:c r="G39" s="24" t="str">
-        <x:v>Mixed approved/proposed</x:v>
+        <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="H39" s="24" t="str">
         <x:v>Yes</x:v>
@@ -28055,7 +28043,7 @@
         <x:v>Use one concise next-step block with owner, explanation and direct action where authorised.</x:v>
       </x:c>
       <x:c r="F42" s="24" t="str">
-        <x:v>KT-STD-001 v1.8 / current module document</x:v>
+        <x:v>KT-STD-001 v1.9 / current module document</x:v>
       </x:c>
       <x:c r="G42" s="24" t="str">
         <x:v>Approved requirement</x:v>
@@ -28103,7 +28091,7 @@
         <x:v>Verify that copy identifies the next actor and correction route without internal jargon.</x:v>
       </x:c>
       <x:c r="F43" s="24" t="str">
-        <x:v>KT-STD-001 v1.8</x:v>
+        <x:v>KT-STD-001 v1.9</x:v>
       </x:c>
       <x:c r="G43" s="24" t="str">
         <x:v>Approved requirement</x:v>
@@ -28151,7 +28139,7 @@
         <x:v>Show work requiring action separately from items waiting on another responsibility.</x:v>
       </x:c>
       <x:c r="F44" s="24" t="str">
-        <x:v>KT-STD-001 v1.8 / PLN-CHG-001 v1.27 / BUD-CHG-001 v1.11 / REQ-CHG-001 v1.12</x:v>
+        <x:v>KT-STD-001 v1.9 / PLN-CHG-001 v1.27 / BUD-CHG-001 v1.11 / REQ-CHG-001 v1.12</x:v>
       </x:c>
       <x:c r="G44" s="24" t="str">
         <x:v>Approved requirement</x:v>
@@ -28199,7 +28187,7 @@
         <x:v>Orient users without duplicating status, exposing internal machinery or overwhelming the primary task.</x:v>
       </x:c>
       <x:c r="F45" s="24" t="str">
-        <x:v>KT-STD-001 v1.8 / current module document</x:v>
+        <x:v>KT-STD-001 v1.9 / current module document</x:v>
       </x:c>
       <x:c r="G45" s="24" t="str">
         <x:v>Approved requirement</x:v>
@@ -32698,7 +32686,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48d787fd50224fd9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5907ce5713b14ae6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38495,7 +38483,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9a2fcbb8c434f84"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d68248dd93d4b50"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38737,22 +38725,22 @@
         <x:v>Approval</x:v>
       </x:c>
       <x:c r="D7" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.11 remains proposed.</x:v>
+        <x:v>TPR-CHG-001 v0.12 approved on 26 September 2026; v0.11 was proposed and never approved.</x:v>
       </x:c>
       <x:c r="E7" s="24" t="str">
-        <x:v>Open</x:v>
+        <x:v>Closed</x:v>
       </x:c>
       <x:c r="F7" s="24" t="str">
         <x:v>Project Owner</x:v>
       </x:c>
       <x:c r="G7" s="24" t="str">
-        <x:v>Complete final cross-document review and approve.</x:v>
+        <x:v>No approval action remains; implementation and verification are tracked separately.</x:v>
       </x:c>
       <x:c r="H7" s="24" t="str">
         <x:v>Authoritative Tender implementation baseline</x:v>
       </x:c>
       <x:c r="I7" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.11 control block</x:v>
+        <x:v>TPR-CHG-001 v0.12 approval control block</x:v>
       </x:c>
       <x:c r="J7" s="2"/>
       <x:c r="K7" s="2"/>
@@ -38783,22 +38771,22 @@
         <x:v>Approval</x:v>
       </x:c>
       <x:c r="D8" s="24" t="str">
-        <x:v>BDS-CHG-001 v0.7 remains proposed.</x:v>
+        <x:v>BDS-CHG-001 v0.8 approved on 26 September 2026; v0.7 was never approved.</x:v>
       </x:c>
       <x:c r="E8" s="24" t="str">
-        <x:v>Open</x:v>
+        <x:v>Closed</x:v>
       </x:c>
       <x:c r="F8" s="24" t="str">
         <x:v>Project Owner</x:v>
       </x:c>
       <x:c r="G8" s="24" t="str">
-        <x:v>Approve after Gate 1 reconciliation.</x:v>
+        <x:v>No further requirement approval for v0.8; retain separate TPR v0.13 dependency and production operating gates.</x:v>
       </x:c>
       <x:c r="H8" s="24" t="str">
-        <x:v>Authoritative Bid Submission implementation baseline</x:v>
+        <x:v>None—requirements approval recorded</x:v>
       </x:c>
       <x:c r="I8" s="24" t="str">
-        <x:v>BDS-CHG-001 v0.7 control block</x:v>
+        <x:v>BDS-CHG-001 v0.8 approval record</x:v>
       </x:c>
       <x:c r="J8" s="2"/>
       <x:c r="K8" s="2"/>
@@ -38829,22 +38817,22 @@
         <x:v>Approval</x:v>
       </x:c>
       <x:c r="D9" s="24" t="str">
-        <x:v>STD-TPL-001 v0.10 remains proposed.</x:v>
+        <x:v>STD-TPL-001 v0.10 was approved by the Project Owner on 26 September 2026.</x:v>
       </x:c>
       <x:c r="E9" s="24" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="F9" s="24" t="str">
         <x:v>Project Owner</x:v>
       </x:c>
       <x:c r="G9" s="24" t="str">
-        <x:v>Approve curation and release standard.</x:v>
+        <x:v>No further document-approval action.</x:v>
       </x:c>
       <x:c r="H9" s="24" t="str">
-        <x:v>Rebuilt response-capable tender bundle</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="I9" s="24" t="str">
-        <x:v>STD-TPL-001 v0.10 control block</x:v>
+        <x:v>STD-TPL-001 v0.10 approval block, 26 September 2026</x:v>
       </x:c>
       <x:c r="J9" s="2"/>
       <x:c r="K9" s="2"/>
@@ -38918,10 +38906,10 @@
         <x:v>Critical</x:v>
       </x:c>
       <x:c r="C11" s="24" t="str">
-        <x:v>Release gate</x:v>
+        <x:v>Bundle readiness</x:v>
       </x:c>
       <x:c r="D11" s="24" t="str">
-        <x:v>The existing IT Equipment bundle is not an approved exact release manifest under STD-TPL-001 v0.10.</x:v>
+        <x:v>The earlier IT Equipment candidate ZIP has not been reconciled and installed as a verified release under amended STD-TPL-001 v0.10.</x:v>
       </x:c>
       <x:c r="E11" s="24" t="str">
         <x:v>Open</x:v>
@@ -38930,13 +38918,13 @@
         <x:v>Controlled release owner</x:v>
       </x:c>
       <x:c r="G11" s="24" t="str">
-        <x:v>Rebuild, verify and approve the exact manifest.</x:v>
+        <x:v>Rebuild and verify the bundle; install with matching assets and renderer, then Administrator may turn it On.</x:v>
       </x:c>
       <x:c r="H11" s="24" t="str">
         <x:v>Tender publication and production Bid Submission</x:v>
       </x:c>
       <x:c r="I11" s="24" t="str">
-        <x:v>STD-TPL-001 v0.10; candidate ZIP</x:v>
+        <x:v>STD-TPL-001 v0.10 in-version amendment; FU-01 OD5; earlier candidate ZIP</x:v>
       </x:c>
       <x:c r="J11" s="2"/>
       <x:c r="K11" s="2"/>
@@ -38982,7 +38970,7 @@
         <x:v>Production submission</x:v>
       </x:c>
       <x:c r="I12" s="24" t="str">
-        <x:v>BDS-CHG-001 v0.7; G1-REG-001 v1.1</x:v>
+        <x:v>BDS-CHG-001 v0.8; G1-REG-001 v1.1</x:v>
       </x:c>
       <x:c r="J12" s="2"/>
       <x:c r="K12" s="2"/>
@@ -39243,7 +39231,7 @@
         <x:v>Cross-module adoption</x:v>
       </x:c>
       <x:c r="D18" s="24" t="str">
-        <x:v>KT-STD-001 v1.8 is approved, but complete implementation evidence for its next-step, guard-reason, hand-off, My Work, Home and no-dead-end contracts does not yet exist across the active modules.</x:v>
+        <x:v>KT-STD-001 v1.9 is approved, but complete implementation evidence for its next-step, guard-reason, hand-off, My Work, Home and no-dead-end contracts does not yet exist across the active modules.</x:v>
       </x:c>
       <x:c r="E18" s="24" t="str">
         <x:v>Open</x:v>
@@ -39258,7 +39246,7 @@
         <x:v>Usability-complete Gate 1 verification</x:v>
       </x:c>
       <x:c r="I18" s="24" t="str">
-        <x:v>KT-STD-001 v1.8; PLN-CHG-001 v1.27; Workflow Guidance Standard</x:v>
+        <x:v>KT-STD-001 v1.9; PLN-CHG-001 v1.27; Workflow Guidance Standard</x:v>
       </x:c>
       <x:c r="J18" s="2"/>
       <x:c r="K18" s="2"/>
@@ -39335,22 +39323,22 @@
         <x:v>Approval</x:v>
       </x:c>
       <x:c r="D20" s="24" t="str">
-        <x:v>STD-TPL-IMP-001 v1.0 is the proposed implementation authority and is not yet approved.</x:v>
+        <x:v>STD-TPL-IMP-001 v1.1 was approved by the Project Owner on 26 September 2026; v1.0 was never approved.</x:v>
       </x:c>
       <x:c r="E20" s="24" t="str">
-        <x:v>Open</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="F20" s="24" t="str">
         <x:v>Project Owner</x:v>
       </x:c>
       <x:c r="G20" s="24" t="str">
-        <x:v>Review and approve with STD-TPL-001 v0.10 before Claude Code implements the template runtime.</x:v>
+        <x:v>Implement v1.1 and reconcile named consumer documents to OD5.</x:v>
       </x:c>
       <x:c r="H20" s="24" t="str">
-        <x:v>Authoritative STD runtime implementation</x:v>
+        <x:v>None for implementation authority; consumer reconciliation remains</x:v>
       </x:c>
       <x:c r="I20" s="24" t="str">
-        <x:v>STD-TPL-IMP-001 v1.0 control block</x:v>
+        <x:v>STD-TPL-IMP-001 v1.1 approval block; Project Owner instruction 26 September 2026</x:v>
       </x:c>
       <x:c r="J20" s="2"/>
       <x:c r="K20" s="2"/>
@@ -44450,7 +44438,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90ea2ab8c6db4a76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R571be035568e463d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(bid-opening): approve BOP-CHG-001 v0.10; plan, tracker and boards for Phase 0
Admits the approved Bid Opening contract (BOP-CHG-001 v0.9 and v0.10),
the approved shared Proceedings contract (PRC-CHG-001 v0.9), the approved
TRUST-ADR-001 v0.1 and KT-STD-001 v1.10, the refreshed register, and the
v0.9.2 artboard pack (50 drawn boards).

Adds the v0.10 implementation plan, tracker, follow-ups, board inventory
and v0.9-to-v0.10 difference record. Drafts KT-STD-001 v1.11 (Proposed)
adding the owner-requested actors Daniel Otieno and Jane Wanjiku to §8.3.

Phase 0 gate BOP-G00. The working-tree deletion of the PRC v0.1/v0.2
drafts is deliberately left out (FU-BOP-13).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/mvp-1-r1/98_work_progress/KenTender_Documentation_Control_Register.xlsx
+++ b/docs/mvp-1-r1/98_work_progress/KenTender_Documentation_Control_Register.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rf03793996ed843ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="2" r:id="R40d4e62b43384dac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interfaces" sheetId="3" r:id="R5c340d2232684845"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R9364b9ae0d004b12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery" sheetId="5" r:id="R264f413469df47da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future Work" sheetId="6" r:id="R7ea02c27ad7848be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="7" r:id="R0bda82e023d34079"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rddb14e0378f34914"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="2" r:id="Rf581a787ea874bcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interfaces" sheetId="3" r:id="R5ef4927187344fab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Raabcad47cdf6478d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery" sheetId="5" r:id="R0ce8146b9b3e41d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future Work" sheetId="6" r:id="Rda6ef2dd99354f21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="7" r:id="R3a6c9235a27649a1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22,7 +22,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="9">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -74,8 +74,13 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF9C0006"/>
+      <x:name val="Aptos"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -112,6 +117,21 @@
         <x:fgColor rgb="FFD9EAF7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -133,7 +153,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="37">
+  <x:cellXfs count="41">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -239,6 +259,18 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top"/>
     </x:xf>
   </x:cellXfs>
@@ -1894,7 +1926,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>Current controlled baseline and delivery status as at 2026-09-26. Requirement approval, implementation, verification and release are tracked independently.</x:v>
+        <x:v>Current controlled baseline and delivery status as at 2026-09-28. Requirement approval, implementation, verification and release are tracked independently.</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -2018,23 +2050,23 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="20" t="n">
-        <x:f>COUNTA(Documents!A6:A29)</x:f>
-        <x:v>24</x:v>
+        <x:f>COUNTA(Documents!A6:A32)</x:f>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="B6" s="20"/>
       <x:c r="C6" s="20" t="n">
-        <x:f>COUNTIF(Documents!F6:F29,"Approved requirement")</x:f>
-        <x:v>12</x:v>
+        <x:f>COUNTIF(Documents!F6:F32,"Approved requirement")</x:f>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D6" s="20"/>
       <x:c r="E6" s="20" t="n">
-        <x:f>COUNTIF(Documents!F6:F29,"Project Owner review")</x:f>
+        <x:f>COUNTIF(Documents!F6:F32,"Project Owner review")</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="F6" s="20"/>
       <x:c r="G6" s="20" t="n">
-        <x:f>COUNTIF(Delivery!I6:I49,"Not started")+COUNTIF(Delivery!I6:I49,"Planned")</x:f>
-        <x:v>44</x:v>
+        <x:f>COUNTIF(Delivery!I6:I51,"Not started")+COUNTIF(Delivery!I6:I51,"Planned")</x:f>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="H6" s="20"/>
       <x:c r="I6" s="2"/>
@@ -8335,7 +8367,7 @@
         <x:v>Tenders</x:v>
       </x:c>
       <x:c r="C12" s="2" t="str">
-        <x:v>0.12</x:v>
+        <x:v>0.13</x:v>
       </x:c>
       <x:c r="D12" s="24" t="str">
         <x:v>Tender Preparation and Publication</x:v>
@@ -8347,10 +8379,10 @@
         <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="G12" s="36" t="n">
-        <x:v>46291</x:v>
+        <x:v>46293</x:v>
       </x:c>
       <x:c r="H12" s="24" t="str">
-        <x:v>v0.11 proposed, never approved</x:v>
+        <x:v>v0.12 approved 26 September 2026; v0.11 proposed, never approved</x:v>
       </x:c>
       <x:c r="I12" s="24" t="str">
         <x:v>Planned</x:v>
@@ -8365,16 +8397,16 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="M12" s="24" t="str">
-        <x:v>Approved Tender preparation, approval, publication, clarifications, addenda, cancellation, bound STD-release lifecycle and KT-STD-001 v1.8 journey guidance.</x:v>
+        <x:v>Approved Tender preparation, approval, publication, clarifications, addenda, cancellation, exact bound STD-release lifecycle including published Superseded/Withdrawn behavior, and KT-STD-001 v1.8 journey guidance.</x:v>
       </x:c>
       <x:c r="N12" s="24" t="str">
-        <x:v>REQ-CHG-001 v1.12; CFG-CHG-002 v0.16; STD-TPL-001 v0.10; STD-TPL-IMP-001 v1.1; BDS-CHG-001 v0.7</x:v>
+        <x:v>REQ-CHG-001 v1.12; CFG-CHG-002 v0.16; STD-TPL-001 v0.10; STD-TPL-IMP-001 v1.1; BDS-CHG-001 v0.8; BOP-CHG-001 v0.10 and PRC-CHG-001 v0.9 proposed for post-close cancellation; Award-status owner pending</x:v>
       </x:c>
       <x:c r="O12" s="24" t="str">
-        <x:v>Implement approved v0.12 and verify §§14–15; new binding requires an intact Available release switched On. Document approval is not production acceptance.</x:v>
+        <x:v>Implement approved v0.13. Proposed v0.14 (KenTender_TPR-CHG-001_Tenders_v0_14_proposed.md; libfile_000ff3f0efe881918a374f6f15819fbb) supplies a guarded post-close cancellation seam but is not approved or enabled. Obtain legal ground mapping and authoritative Award-status integration before approval/release.</x:v>
       </x:c>
       <x:c r="P12" s="24" t="str">
-        <x:v>https://chatgpt.com/api/library/files/libfile_357a5c0bfd8881918423b65cb452bd41/download</x:v>
+        <x:v>https://chatgpt.com/api/library/files/libfile_6aaf080652a08191a8796a086f31b59c/download</x:v>
       </x:c>
       <x:c r="Q12" s="2"/>
       <x:c r="R12" s="2"/>
@@ -8428,10 +8460,10 @@
         <x:v>Public discovery, supplier Account, structured Goods/IT bid preparation, signature, receipt, replacement and sealed Bid Opening handoff, with actor-specific guidance and bound STD-release controls.</x:v>
       </x:c>
       <x:c r="N13" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.12; STD-TPL-001 v0.10; STD-TPL-IMP-001 v1.1; CFG-CHG-002 v0.16; AUTH-ADR-001 v1.10; KT-STD-001 v1.8; G1-REG-001 v1.1</x:v>
+        <x:v>TPR-CHG-001 v0.13; STD-TPL-001 v0.10; STD-TPL-IMP-001 v1.1; CFG-CHG-002 v0.16; AUTH-ADR-001 v1.10; KT-STD-001 v1.8; G1-REG-001 v1.1</x:v>
       </x:c>
       <x:c r="O13" s="24" t="str">
-        <x:v>Implement approved v0.8; keep production submission disabled until §§5.10 and 15 gates pass. Published-Tender Superseded/Withdrawn behavior remains conditional on approval of TPR-CHG-001 v0.13. Reconcile its §10 presentation with the newly approved KT-STD-001 v1.9 before design execution.</x:v>
+        <x:v>Implement approved v0.8 with production disabled until §§5.10 and 15 gates pass; TPR v0.13 is approved. Proposed BDS v0.9 (libfile_f8038abb4ed08191983a122d03a31c1f) corrects the pre-opening physical-security receipt owner visibility conflict and stale TPR conditions; v0.8 remains normative pending v0.9 approval.</x:v>
       </x:c>
       <x:c r="P13" s="24" t="str">
         <x:v>https://chatgpt.com/api/library/files/libfile_7252e90793e4819199bca1d68fab4457/download</x:v>
@@ -8575,7 +8607,7 @@
         <x:v>Document, Design and Verification Standards</x:v>
       </x:c>
       <x:c r="C16" s="2" t="str">
-        <x:v>1.9</x:v>
+        <x:v>1.10</x:v>
       </x:c>
       <x:c r="D16" s="24" t="str">
         <x:v>All</x:v>
@@ -8587,10 +8619,10 @@
         <x:v>Approved requirement</x:v>
       </x:c>
       <x:c r="G16" s="36" t="n">
-        <x:v>46291</x:v>
+        <x:v>46294</x:v>
       </x:c>
       <x:c r="H16" s="24" t="str">
-        <x:v>v1.8 approved 25 September 2026; v1.7 and earlier remain historical evidence</x:v>
+        <x:v>v1.9 approved 26 September 2026, retained as historical evidence</x:v>
       </x:c>
       <x:c r="I16" s="24" t="str">
         <x:v>Not applicable</x:v>
@@ -8605,16 +8637,16 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="M16" s="24" t="str">
-        <x:v>Current cross-cutting design and verification authority. Refines the white page sheet, guidance-region placement and restrained accent rules; retains the v1.8 next-step, journey, guard-reason, hand-off, My Work, Home and dead-end conformance contracts.</x:v>
+        <x:v>Current cross-cutting standard, including plain language, minimum steps, Scheduled next step and actor/state/event conformance; retains earlier design and verification rules.</x:v>
       </x:c>
       <x:c r="N16" s="24" t="str">
         <x:v>Workflow Guidance Standard; all controlled change documents</x:v>
       </x:c>
       <x:c r="O16" s="24" t="str">
-        <x:v>Apply v1.9 to every new or revised change unit and artboard prompt; retain the v1.8 runtime and verification contracts carried forward into v1.9.</x:v>
+        <x:v>Apply approved v1.10 to future and revised design contracts: plain language, minimum steps, Scheduled next step and actor/state/event conformance.</x:v>
       </x:c>
       <x:c r="P16" s="24" t="str">
-        <x:v>https://chatgpt.com/api/library/files/libfile_c189a864c48c81918002bab99a3dc04c/download</x:v>
+        <x:v>https://chatgpt.com/api/library/files/libfile_17ffb496b8708191bfba06c99365e11c/download</x:v>
       </x:c>
       <x:c r="Q16" s="2"/>
       <x:c r="R16" s="2"/>
@@ -9372,22 +9404,52 @@
       <x:c r="Z29" s="2"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="2"/>
-      <x:c r="B30" s="2"/>
-      <x:c r="C30" s="2"/>
-      <x:c r="D30" s="2"/>
-      <x:c r="E30" s="2"/>
-      <x:c r="F30" s="2"/>
-      <x:c r="G30" s="2"/>
-      <x:c r="H30" s="2"/>
-      <x:c r="I30" s="2"/>
-      <x:c r="J30" s="2"/>
-      <x:c r="K30" s="2"/>
-      <x:c r="L30" s="2"/>
-      <x:c r="M30" s="2"/>
-      <x:c r="N30" s="2"/>
-      <x:c r="O30" s="2"/>
-      <x:c r="P30" s="2"/>
+      <x:c r="A30" s="2" t="str">
+        <x:v>TRUST-ADR-001</x:v>
+      </x:c>
+      <x:c r="B30" s="2" t="str">
+        <x:v>Shared Signing and Sealed Custody</x:v>
+      </x:c>
+      <x:c r="C30" s="2" t="str">
+        <x:v>0.1</x:v>
+      </x:c>
+      <x:c r="D30" s="2" t="str">
+        <x:v>Shared Trust Infrastructure</x:v>
+      </x:c>
+      <x:c r="E30" s="2" t="str">
+        <x:v>Architecture decision</x:v>
+      </x:c>
+      <x:c r="F30" s="37" t="str">
+        <x:v>Approved requirement</x:v>
+      </x:c>
+      <x:c r="G30" s="36" t="n">
+        <x:v>46292</x:v>
+      </x:c>
+      <x:c r="H30" s="2" t="str"/>
+      <x:c r="I30" s="2" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="J30" s="2" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="K30" s="40" t="str">
+        <x:v>Blocked</x:v>
+      </x:c>
+      <x:c r="L30" s="2" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M30" s="2" t="str">
+        <x:v>Locks two distinct signing/decision semantics and separate multi-person sealed-bid custody, defers actual production mechanisms to a shared support module, and permits synthetic test proxies only.</x:v>
+      </x:c>
+      <x:c r="N30" s="2" t="str">
+        <x:v>BDS-CHG-001 v0.8 (v0.9 proposed); BOP-CHG-001 v0.10 proposed; PRC-CHG-001 v0.9 proposed; LAW-V-001</x:v>
+      </x:c>
+      <x:c r="O30" s="2" t="str">
+        <x:v>Approved v0.1 remains architecture authority. Its static Consumers row cites historical BOP v0.1/PRC v0.2; update by a later controlled revision. Test infrastructure administrator is outside proxy confidentiality guarantee. Production support module and operating profile remain separate.</x:v>
+      </x:c>
+      <x:c r="P30" s="2" t="str">
+        <x:v>https://chatgpt.com/api/library/files/libfile_d1eb23c985808191b4a6e33a29af86b5/download</x:v>
+      </x:c>
       <x:c r="Q30" s="2"/>
       <x:c r="R30" s="2"/>
       <x:c r="S30" s="2"/>
@@ -9400,22 +9462,54 @@
       <x:c r="Z30" s="2"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="2"/>
-      <x:c r="B31" s="2"/>
-      <x:c r="C31" s="2"/>
-      <x:c r="D31" s="2"/>
-      <x:c r="E31" s="2"/>
-      <x:c r="F31" s="2"/>
-      <x:c r="G31" s="2"/>
-      <x:c r="H31" s="2"/>
-      <x:c r="I31" s="2"/>
-      <x:c r="J31" s="2"/>
-      <x:c r="K31" s="2"/>
-      <x:c r="L31" s="2"/>
-      <x:c r="M31" s="2"/>
-      <x:c r="N31" s="2"/>
-      <x:c r="O31" s="2"/>
-      <x:c r="P31" s="2"/>
+      <x:c r="A31" s="2" t="str">
+        <x:v>BOP-CHG-001</x:v>
+      </x:c>
+      <x:c r="B31" s="2" t="str">
+        <x:v>Electronic Bid Opening</x:v>
+      </x:c>
+      <x:c r="C31" s="2" t="str">
+        <x:v>0.10</x:v>
+      </x:c>
+      <x:c r="D31" s="2" t="str">
+        <x:v>Bid Opening</x:v>
+      </x:c>
+      <x:c r="E31" s="2" t="str">
+        <x:v>Module requirements</x:v>
+      </x:c>
+      <x:c r="F31" s="38" t="str">
+        <x:v>Approved requirement</x:v>
+      </x:c>
+      <x:c r="G31" s="36" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="H31" s="2" t="str">
+        <x:v>v0.9 approved 29 September 2026, retained as historical evidence</x:v>
+      </x:c>
+      <x:c r="I31" s="2" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="J31" s="2" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="K31" s="40" t="str">
+        <x:v>Not approved</x:v>
+      </x:c>
+      <x:c r="L31" s="2" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M31" s="2" t="str">
+        <x:v>Approved design and development contract. v0.10 adds the opening-access-unavailable scenario, four completed-record correction kinds, the AO Your turn state and a unified Tender route.</x:v>
+      </x:c>
+      <x:c r="N31" s="2" t="str">
+        <x:v>KT-STD-001 v1.10 approved; TPR-CHG-001 v0.13 approved (v0.14 post-close seam proposed); BDS-CHG-001 v0.8 approved (v0.9 correction proposed); PRC-CHG-001 v0.9 approved; TRUST-ADR-001 v0.1 approved; LAW-V-001; future Evaluation intake</x:v>
+      </x:c>
+      <x:c r="O31" s="2" t="str">
+        <x:v>Implement approved v0.10 under KT-STD-001 v1.10 with PRC v0.9. Preserve deferred signing/custody support and the separate TPR v0.14 dependency.</x:v>
+      </x:c>
+      <x:c r="P31" s="2" t="str">
+        <x:v>https://chatgpt.com/api/library/files/libfile_a398ef6e43f08191981ed3372ee79e29/download</x:v>
+      </x:c>
       <x:c r="Q31" s="2"/>
       <x:c r="R31" s="2"/>
       <x:c r="S31" s="2"/>
@@ -9428,22 +9522,54 @@
       <x:c r="Z31" s="2"/>
     </x:row>
     <x:row r="32">
-      <x:c r="A32" s="2"/>
-      <x:c r="B32" s="2"/>
-      <x:c r="C32" s="2"/>
-      <x:c r="D32" s="2"/>
-      <x:c r="E32" s="2"/>
-      <x:c r="F32" s="2"/>
-      <x:c r="G32" s="2"/>
-      <x:c r="H32" s="2"/>
-      <x:c r="I32" s="2"/>
-      <x:c r="J32" s="2"/>
-      <x:c r="K32" s="2"/>
-      <x:c r="L32" s="2"/>
-      <x:c r="M32" s="2"/>
-      <x:c r="N32" s="2"/>
-      <x:c r="O32" s="2"/>
-      <x:c r="P32" s="2"/>
+      <x:c r="A32" s="2" t="str">
+        <x:v>PRC-CHG-001</x:v>
+      </x:c>
+      <x:c r="B32" s="2" t="str">
+        <x:v>Minimal Procurement Proceedings</x:v>
+      </x:c>
+      <x:c r="C32" s="2" t="str">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="D32" s="2" t="str">
+        <x:v>Procurement Proceedings</x:v>
+      </x:c>
+      <x:c r="E32" s="2" t="str">
+        <x:v>Module requirements</x:v>
+      </x:c>
+      <x:c r="F32" s="38" t="str">
+        <x:v>Approved requirement</x:v>
+      </x:c>
+      <x:c r="G32" s="36" t="n">
+        <x:v>46294</x:v>
+      </x:c>
+      <x:c r="H32" s="2" t="str">
+        <x:v>v0.8 proposed, retained; earlier proposals historical; v0.1 accepted scope</x:v>
+      </x:c>
+      <x:c r="I32" s="2" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="J32" s="2" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="K32" s="40" t="str">
+        <x:v>Not approved</x:v>
+      </x:c>
+      <x:c r="L32" s="2" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M32" s="2" t="str">
+        <x:v>Approved minimal shared service bound to BOP v0.10: attributed pre-session arrivals carried into actual session view, owner events, versioned opening record, personal target proof, one-action empty outcome and terminal partial/never-held records. No standalone UI.</x:v>
+      </x:c>
+      <x:c r="N32" s="2" t="str">
+        <x:v>BOP-CHG-001 v0.10 approved; KT-STD-001 v1.10 approved; TPR-CHG-001 v0.13 approved (v0.14 proposed); TRUST-ADR-001 v0.1 approved; LAW-V-001</x:v>
+      </x:c>
+      <x:c r="O32" s="2" t="str">
+        <x:v>Implement approved v0.9 with BOP v0.10 under KT-STD-001 v1.10. Preserve the deferred shared signing/custody integration.</x:v>
+      </x:c>
+      <x:c r="P32" s="2" t="str">
+        <x:v>https://chatgpt.com/api/library/files/libfile_e3c0b33a03448191b9463fc13f4a9c0f/download</x:v>
+      </x:c>
       <x:c r="Q32" s="2"/>
       <x:c r="R32" s="2"/>
       <x:c r="S32" s="2"/>
@@ -14210,7 +14336,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R71655390f1ff431c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44663dcb7900455e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14602,7 +14728,7 @@
         <x:v>Not evidenced</x:v>
       </x:c>
       <x:c r="H10" s="24" t="str">
-        <x:v>REQ-CHG-001 v1.12 / TPR-CHG-001 v0.12</x:v>
+        <x:v>REQ-CHG-001 v1.12 / TPR-CHG-001 v0.13</x:v>
       </x:c>
       <x:c r="I10" s="24" t="str">
         <x:v>Tender creation must reject missing, stale or unauthorised handoff data.</x:v>
@@ -14740,7 +14866,7 @@
         <x:v>Not evidenced</x:v>
       </x:c>
       <x:c r="H13" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.12 / BDS-CHG-001 v0.8 / STD-TPL-IMP-001 v1.1</x:v>
+        <x:v>TPR-CHG-001 v0.13 / BDS-CHG-001 v0.8 / STD-TPL-IMP-001 v1.1</x:v>
       </x:c>
       <x:c r="I13" s="24" t="str">
         <x:v>Bid UI must be generated only by the shared compiler from the exact effective published definition and release identity.</x:v>
@@ -14786,7 +14912,7 @@
         <x:v>Not evidenced</x:v>
       </x:c>
       <x:c r="H14" s="24" t="str">
-        <x:v>BDS-CHG-001 v0.8 / TPR-CHG-001 v0.12</x:v>
+        <x:v>BDS-CHG-001 v0.8 / TPR-CHG-001 v0.13</x:v>
       </x:c>
       <x:c r="I14" s="24" t="str">
         <x:v>Start bid must not create a half-registered candidate or orphan question.</x:v>
@@ -14970,7 +15096,7 @@
         <x:v>Not evidenced</x:v>
       </x:c>
       <x:c r="H18" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.12 / BDS-CHG-001 v0.8</x:v>
+        <x:v>TPR-CHG-001 v0.13 / BDS-CHG-001 v0.8</x:v>
       </x:c>
       <x:c r="I18" s="24" t="str">
         <x:v>Changed requirements require an issued addendum; clarifications alone cannot mutate the bid definition.</x:v>
@@ -15016,7 +15142,7 @@
         <x:v>Not evidenced</x:v>
       </x:c>
       <x:c r="H19" s="24" t="str">
-        <x:v>STD-TPL-001 v0.10 / STD-TPL-IMP-001 v1.1 / TPR-CHG-001 v0.12</x:v>
+        <x:v>STD-TPL-001 v0.10 / STD-TPL-IMP-001 v1.1 / TPR-CHG-001 v0.13</x:v>
       </x:c>
       <x:c r="I19" s="24" t="str">
         <x:v>New binding requires site On and valid integrity/renderer; Off preserves existing bindings, safety/legal withdrawal blocks affected unpublished publication; never automatically rebind.</x:v>
@@ -15086,15 +15212,33 @@
       <x:c r="Z20" s="2"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="2"/>
-      <x:c r="B21" s="2"/>
-      <x:c r="C21" s="2"/>
-      <x:c r="D21" s="2"/>
-      <x:c r="E21" s="2"/>
-      <x:c r="F21" s="2"/>
-      <x:c r="G21" s="2"/>
-      <x:c r="H21" s="2"/>
-      <x:c r="I21" s="2"/>
+      <x:c r="A21" s="2" t="str">
+        <x:v>IF-016</x:v>
+      </x:c>
+      <x:c r="B21" s="2" t="str">
+        <x:v>Trust, Signing and Custody</x:v>
+      </x:c>
+      <x:c r="C21" s="2" t="str">
+        <x:v>BDS / BOP / PRC</x:v>
+      </x:c>
+      <x:c r="D21" s="2" t="str">
+        <x:v>Exact-target signature verification and sealed bid deposit/opening custody with authoritative receipts and independent member authorization</x:v>
+      </x:c>
+      <x:c r="E21" s="2" t="str">
+        <x:v>Deferred production contract; test proxy approved</x:v>
+      </x:c>
+      <x:c r="F21" s="2" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="G21" s="2" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="H21" s="2" t="str">
+        <x:v>TRUST-ADR-001 v0.1; BDS-CHG-001 v0.8; BOP-CHG-001 v0.1; PRC-CHG-001 v0.2</x:v>
+      </x:c>
+      <x:c r="I21" s="2" t="str">
+        <x:v>No production submission/opening/signature on absent or uncertain trust/custody result. A synthetic proxy cannot turn the default-false BDS gate on.</x:v>
+      </x:c>
       <x:c r="J21" s="2"/>
       <x:c r="K21" s="2"/>
       <x:c r="L21" s="2"/>
@@ -20165,7 +20309,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R02c7118153cc4ed9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R616750a2f016462e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21302,12 +21446,24 @@
       <x:c r="Z29" s="2"/>
     </x:row>
     <x:row r="30">
-      <x:c r="A30" s="2"/>
-      <x:c r="B30" s="2"/>
-      <x:c r="C30" s="2"/>
-      <x:c r="D30" s="2"/>
-      <x:c r="E30" s="2"/>
-      <x:c r="F30" s="2"/>
+      <x:c r="A30" s="2" t="str">
+        <x:v>DEC-025</x:v>
+      </x:c>
+      <x:c r="B30" s="2" t="str">
+        <x:v>Keep ordinary authenticated workflow decisions distinct from statutory advanced electronic signatures; defer actual signing to the shared Trust, Signing and Custody support module.</x:v>
+      </x:c>
+      <x:c r="C30" s="2" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="D30" s="2" t="str">
+        <x:v>TRUST-ADR-001 v0.1, 2026-09-27</x:v>
+      </x:c>
+      <x:c r="E30" s="2" t="str">
+        <x:v>Exact-target, per-member test attestations allowed only with synthetic data and explicit test labels; real signing requires personal provider evidence and legal page/initial mapping.</x:v>
+      </x:c>
+      <x:c r="F30" s="2" t="str">
+        <x:v>Show Test attestation in test profile; no generic approval as a signature.</x:v>
+      </x:c>
       <x:c r="G30" s="2"/>
       <x:c r="H30" s="2"/>
       <x:c r="I30" s="2"/>
@@ -21330,12 +21486,24 @@
       <x:c r="Z30" s="2"/>
     </x:row>
     <x:row r="31">
-      <x:c r="A31" s="2"/>
-      <x:c r="B31" s="2"/>
-      <x:c r="C31" s="2"/>
-      <x:c r="D31" s="2"/>
-      <x:c r="E31" s="2"/>
-      <x:c r="F31" s="2"/>
+      <x:c r="A31" s="2" t="str">
+        <x:v>DEC-026</x:v>
+      </x:c>
+      <x:c r="B31" s="2" t="str">
+        <x:v>Keep sealed-bid custody and multi-person opening release independent of chair/admin authority; defer real keys, provider and threshold to shared infrastructure.</x:v>
+      </x:c>
+      <x:c r="C31" s="2" t="str">
+        <x:v>Approved</x:v>
+      </x:c>
+      <x:c r="D31" s="2" t="str">
+        <x:v>TRUST-ADR-001 v0.1, 2026-09-27</x:v>
+      </x:c>
+      <x:c r="E31" s="2" t="str">
+        <x:v>Synthetic tender-box and two-person test release may exercise ceremony; BDS production submission flag stays false and BOP production disabled until verified real services.</x:v>
+      </x:c>
+      <x:c r="F31" s="2" t="str">
+        <x:v>Visible test-environment status and honest unavailable production guidance; no proxy receipt as a live Submitted bid.</x:v>
+      </x:c>
       <x:c r="G31" s="2"/>
       <x:c r="H31" s="2"/>
       <x:c r="I31" s="2"/>
@@ -26107,7 +26275,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09de1e094824414d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b9767b4cdac4179"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26555,7 +26723,7 @@
         <x:v>Name the source problem and owner without technical codes.</x:v>
       </x:c>
       <x:c r="F11" s="24" t="str">
-        <x:v>REQ-CHG-001 v1.12 / TPR-CHG-001 v0.12</x:v>
+        <x:v>REQ-CHG-001 v1.12 / TPR-CHG-001 v0.13</x:v>
       </x:c>
       <x:c r="G11" s="24" t="str">
         <x:v>Approved requirement</x:v>
@@ -26603,7 +26771,7 @@
         <x:v>Progressive preparation journey with concise supporting detail.</x:v>
       </x:c>
       <x:c r="F12" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.12 / STD-TPL-001 v0.10</x:v>
+        <x:v>TPR-CHG-001 v0.13 / STD-TPL-001 v0.10</x:v>
       </x:c>
       <x:c r="G12" s="24" t="str">
         <x:v>Approved requirement</x:v>
@@ -26651,7 +26819,7 @@
         <x:v>Clear confirmed/evidence-required states and direct actions.</x:v>
       </x:c>
       <x:c r="F13" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.12</x:v>
+        <x:v>TPR-CHG-001 v0.13</x:v>
       </x:c>
       <x:c r="G13" s="24" t="str">
         <x:v>Approved requirement</x:v>
@@ -26699,7 +26867,7 @@
         <x:v>One understandable clarification feed.</x:v>
       </x:c>
       <x:c r="F14" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.12 / BDS-CHG-001 v0.8</x:v>
+        <x:v>TPR-CHG-001 v0.13 / BDS-CHG-001 v0.8</x:v>
       </x:c>
       <x:c r="G14" s="24" t="str">
         <x:v>Approved requirement</x:v>
@@ -26747,7 +26915,7 @@
         <x:v>Prominent change notice and acknowledgement state.</x:v>
       </x:c>
       <x:c r="F15" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.12 / BDS-CHG-001 v0.8</x:v>
+        <x:v>TPR-CHG-001 v0.13 / BDS-CHG-001 v0.8</x:v>
       </x:c>
       <x:c r="G15" s="24" t="str">
         <x:v>Approved requirement</x:v>
@@ -26795,7 +26963,7 @@
         <x:v>Simple search/list/detail; reusable framework pages where suitable.</x:v>
       </x:c>
       <x:c r="F16" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.12 / BDS-CHG-001 v0.8</x:v>
+        <x:v>TPR-CHG-001 v0.13 / BDS-CHG-001 v0.8</x:v>
       </x:c>
       <x:c r="G16" s="24" t="str">
         <x:v>Approved requirement</x:v>
@@ -27659,7 +27827,7 @@
         <x:v>Show successor notice and preserved exact release.</x:v>
       </x:c>
       <x:c r="F34" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.12 / STD-TPL-001 v0.10</x:v>
+        <x:v>TPR-CHG-001 v0.13 / STD-TPL-001 v0.10</x:v>
       </x:c>
       <x:c r="G34" s="24" t="str">
         <x:v>Approved requirement</x:v>
@@ -27707,7 +27875,7 @@
         <x:v>Direct reason, release link and governed next step.</x:v>
       </x:c>
       <x:c r="F35" s="24" t="str">
-        <x:v>TPR-CHG-001 v0.12 / STD-TPL-001 v0.10</x:v>
+        <x:v>TPR-CHG-001 v0.13 / STD-TPL-001 v0.10</x:v>
       </x:c>
       <x:c r="G35" s="24" t="str">
         <x:v>Approved requirement</x:v>
@@ -27899,7 +28067,7 @@
         <x:v>Show concise confirmed treatment with correction route.</x:v>
       </x:c>
       <x:c r="F39" s="24" t="str">
-        <x:v>REQ-CHG-001 v1.12 / TPR-CHG-001 v0.12 / BDS-CHG-001 v0.8</x:v>
+        <x:v>REQ-CHG-001 v1.12 / TPR-CHG-001 v0.13 / BDS-CHG-001 v0.8</x:v>
       </x:c>
       <x:c r="G39" s="24" t="str">
         <x:v>Approved requirement</x:v>
@@ -28411,16 +28579,36 @@
       <x:c r="Z49" s="2"/>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="2"/>
-      <x:c r="B50" s="2"/>
-      <x:c r="C50" s="2"/>
-      <x:c r="D50" s="2"/>
-      <x:c r="E50" s="2"/>
-      <x:c r="F50" s="2"/>
-      <x:c r="G50" s="2"/>
-      <x:c r="H50" s="2"/>
-      <x:c r="I50" s="2"/>
-      <x:c r="J50" s="2"/>
+      <x:c r="A50" s="2" t="str">
+        <x:v>TRUST-001</x:v>
+      </x:c>
+      <x:c r="B50" s="2" t="str">
+        <x:v>Shared Trust Infrastructure</x:v>
+      </x:c>
+      <x:c r="C50" s="2" t="str">
+        <x:v>Build synthetic signing/custody test adapters and later a separately approved production support module.</x:v>
+      </x:c>
+      <x:c r="D50" s="2" t="str">
+        <x:v>Preserve exact-target member evidence, sealed receipts and BOP ordered reveal API; then integrate licensed provider, external keys, independent multi-person release and recovery.</x:v>
+      </x:c>
+      <x:c r="E50" s="2" t="str">
+        <x:v>Keep ordinary approvals and statutory signatures distinct; label test attestations/receipts and hide production submission/opening actions.</x:v>
+      </x:c>
+      <x:c r="F50" s="2" t="str">
+        <x:v>TRUST-ADR-001 v0.1 / BDS-CHG-001 v0.8 / BOP-CHG-001 v0.1 / PRC-CHG-001 v0.2</x:v>
+      </x:c>
+      <x:c r="G50" s="2" t="str">
+        <x:v>Approved requirement</x:v>
+      </x:c>
+      <x:c r="H50" s="2" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="I50" s="2" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="J50" s="2" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
       <x:c r="K50" s="2"/>
       <x:c r="L50" s="2"/>
       <x:c r="M50" s="2"/>
@@ -28439,16 +28627,36 @@
       <x:c r="Z50" s="2"/>
     </x:row>
     <x:row r="51">
-      <x:c r="A51" s="2"/>
-      <x:c r="B51" s="2"/>
-      <x:c r="C51" s="2"/>
-      <x:c r="D51" s="2"/>
-      <x:c r="E51" s="2"/>
-      <x:c r="F51" s="2"/>
-      <x:c r="G51" s="2"/>
-      <x:c r="H51" s="2"/>
-      <x:c r="I51" s="2"/>
-      <x:c r="J51" s="2"/>
+      <x:c r="A51" s="2" t="str">
+        <x:v>G1-031</x:v>
+      </x:c>
+      <x:c r="B51" s="2" t="str">
+        <x:v>Tenders / Bid Submission</x:v>
+      </x:c>
+      <x:c r="C51" s="2" t="str">
+        <x:v>Apply approved published-Tender bound-release behavior after Supersession or Withdrawal.</x:v>
+      </x:c>
+      <x:c r="D51" s="2" t="str">
+        <x:v>Allow already-bound published Tenders on a Superseded release to issue lawful addenda and accept Bid start/submission while exact checks pass; on Withdrawn block new start/addendum/submission/replacement but preserve reads, existing receipts and lawful pre-deadline withdrawal.</x:v>
+      </x:c>
+      <x:c r="E51" s="2" t="str">
+        <x:v>Show truthful lifecycle notices and allowed next actions to internal and supplier users.</x:v>
+      </x:c>
+      <x:c r="F51" s="2" t="str">
+        <x:v>TPR-CHG-001 v0.13 / BDS-CHG-001 v0.8</x:v>
+      </x:c>
+      <x:c r="G51" s="2" t="str">
+        <x:v>Approved requirement</x:v>
+      </x:c>
+      <x:c r="H51" s="2" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="I51" s="2" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="J51" s="2" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
       <x:c r="K51" s="2"/>
       <x:c r="L51" s="2"/>
       <x:c r="M51" s="2"/>
@@ -32686,7 +32894,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5907ce5713b14ae6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00da4d46689f4e68"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33285,14 +33493,28 @@
       <x:c r="Y15" s="2"/>
       <x:c r="Z15" s="2"/>
     </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="2"/>
-      <x:c r="B16" s="2"/>
-      <x:c r="C16" s="2"/>
-      <x:c r="D16" s="2"/>
-      <x:c r="E16" s="2"/>
-      <x:c r="F16" s="2"/>
-      <x:c r="G16" s="2"/>
+    <x:row r="16" ht="80" customHeight="1">
+      <x:c r="A16" s="24" t="str">
+        <x:v>FW-011</x:v>
+      </x:c>
+      <x:c r="B16" s="24" t="str">
+        <x:v>Default internal read access to current Strategy</x:v>
+      </x:c>
+      <x:c r="C16" s="24" t="str">
+        <x:v>Next access-policy revision</x:v>
+      </x:c>
+      <x:c r="D16" s="24" t="str">
+        <x:v>STR-CHG-001 v1.8; AUTH-ADR-001 effective baseline</x:v>
+      </x:c>
+      <x:c r="E16" s="24" t="str">
+        <x:v>To do</x:v>
+      </x:c>
+      <x:c r="F16" s="24" t="str">
+        <x:v>Review access for enabled internal users to Active Strategy data only. Current assignment-based restrictions remain in force; no Draft, submitted review, approval-task, supplier or public access is approved by this entry.</x:v>
+      </x:c>
+      <x:c r="G16" s="24" t="str">
+        <x:v>Decide baseline read policy versus per-module Reader responsibility; revise STR and AUTH through controlled versions; verify list, detail, export, API and write boundaries.</x:v>
+      </x:c>
       <x:c r="H16" s="2"/>
       <x:c r="I16" s="2"/>
       <x:c r="J16" s="2"/>
@@ -33314,13 +33536,27 @@
       <x:c r="Z16" s="2"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="2"/>
-      <x:c r="B17" s="2"/>
-      <x:c r="C17" s="2"/>
-      <x:c r="D17" s="2"/>
-      <x:c r="E17" s="2"/>
-      <x:c r="F17" s="2"/>
-      <x:c r="G17" s="2"/>
+      <x:c r="A17" s="2" t="str">
+        <x:v>FW-012</x:v>
+      </x:c>
+      <x:c r="B17" s="2" t="str">
+        <x:v>Production Trust, Signing and Sealed Custody support module</x:v>
+      </x:c>
+      <x:c r="C17" s="2" t="str">
+        <x:v>Later support-module version</x:v>
+      </x:c>
+      <x:c r="D17" s="2" t="str">
+        <x:v>TRUST-ADR-001 v0.1; licensed/accredited provider; legal L1/L2; approved government operating profile; production-equivalent tests</x:v>
+      </x:c>
+      <x:c r="E17" s="2" t="str">
+        <x:v>Planned</x:v>
+      </x:c>
+      <x:c r="F17" s="2" t="str">
+        <x:v>Only synthetic, explicitly labelled test proxies now. BDS v0.8 production bid submission remains disabled and electronic Bid Opening cannot be used for real bids.</x:v>
+      </x:c>
+      <x:c r="G17" s="2" t="str">
+        <x:v>Approve provider/signing method, per-target legal equivalence, custody/key threshold, credentials, recovery, external channel and test/release evidence.</x:v>
+      </x:c>
       <x:c r="H17" s="2"/>
       <x:c r="I17" s="2"/>
       <x:c r="J17" s="2"/>
@@ -38483,7 +38719,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d68248dd93d4b50"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R998d104da2ab441a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -39405,15 +39641,33 @@
       <x:c r="Z21" s="2"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="2"/>
-      <x:c r="B22" s="2"/>
-      <x:c r="C22" s="2"/>
-      <x:c r="D22" s="2"/>
-      <x:c r="E22" s="2"/>
-      <x:c r="F22" s="2"/>
-      <x:c r="G22" s="2"/>
-      <x:c r="H22" s="2"/>
-      <x:c r="I22" s="2"/>
+      <x:c r="A22" s="2" t="str">
+        <x:v>AUD-017</x:v>
+      </x:c>
+      <x:c r="B22" s="2" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="C22" s="2" t="str">
+        <x:v>Cross-document reconciliation</x:v>
+      </x:c>
+      <x:c r="D22" s="2" t="str">
+        <x:v>BDS v0.8 physical-security receipt view discloses supplier identity before opening despite a blanket no-PE-bidder-identity statement; BOP v0.1 and PRC v0.2 lacked closed ceremony/PRC bindings. Controlled BOP v0.2, PRC v0.3 and BDS v0.9 are proposed corrections.</x:v>
+      </x:c>
+      <x:c r="E22" s="2" t="str">
+        <x:v>Open</x:v>
+      </x:c>
+      <x:c r="F22" s="2" t="str">
+        <x:v>Project Owner / requirements owner</x:v>
+      </x:c>
+      <x:c r="G22" s="2" t="str">
+        <x:v>Review the three coordinated proposals; approve BDS receipt-owner exception and BOP/PRC lifecycle, then close actual renderer/proof and lawful operating-profile gates separately.</x:v>
+      </x:c>
+      <x:c r="H22" s="2" t="str">
+        <x:v>Reconciled Bid Opening design and production authority</x:v>
+      </x:c>
+      <x:c r="I22" s="2" t="str">
+        <x:v>BDS v0.8 §§5.9, 10.16; BOP v0.2 §7.1; PRC v0.3 §7.1; BDS v0.9 §12.2A</x:v>
+      </x:c>
       <x:c r="J22" s="2"/>
       <x:c r="K22" s="2"/>
       <x:c r="L22" s="2"/>
@@ -39433,15 +39687,33 @@
       <x:c r="Z22" s="2"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23" s="2"/>
-      <x:c r="B23" s="2"/>
-      <x:c r="C23" s="2"/>
-      <x:c r="D23" s="2"/>
-      <x:c r="E23" s="2"/>
-      <x:c r="F23" s="2"/>
-      <x:c r="G23" s="2"/>
-      <x:c r="H23" s="2"/>
-      <x:c r="I23" s="2"/>
+      <x:c r="A23" s="2" t="str">
+        <x:v>AUD-018</x:v>
+      </x:c>
+      <x:c r="B23" s="2" t="str">
+        <x:v>High</x:v>
+      </x:c>
+      <x:c r="C23" s="2" t="str">
+        <x:v>Design closure</x:v>
+      </x:c>
+      <x:c r="D23" s="2" t="str">
+        <x:v>Earlier BOP/PRC versions conflated design fixtures with live evidence, contained contradictory actor/branch events, and left visible actions without a clear owner command. Approved BOP v0.10 and PRC v0.9 provide the end-to-end matrix, corrected branches, owner bindings and repeatable mechanical check. The cross-project standard gate is approved in KT-STD-001 v1.10.</x:v>
+      </x:c>
+      <x:c r="E23" s="2" t="str">
+        <x:v>Controlled</x:v>
+      </x:c>
+      <x:c r="F23" s="2" t="str">
+        <x:v>Requirements owner / Project Owner</x:v>
+      </x:c>
+      <x:c r="G23" s="2" t="str">
+        <x:v>Apply approved BOP v0.10 / PRC v0.9 and KT-STD-001 v1.10, approved 29 September 2026. Use direct copy comparisons and actor/state/event review on affected branches. TPR v0.14 post-close cancellation remains a separately owned dependency.</x:v>
+      </x:c>
+      <x:c r="H23" s="2" t="str">
+        <x:v>No BOP artboard; real opening activation and integrated proof remain separate later decisions</x:v>
+      </x:c>
+      <x:c r="I23" s="2" t="str">
+        <x:v>Approved BOP v0.10, admitted 29 September 2026; approved PRC v0.9 and KT-STD-001 v1.10. BOP v0.9 retained as the prior approved baseline.</x:v>
+      </x:c>
       <x:c r="J23" s="2"/>
       <x:c r="K23" s="2"/>
       <x:c r="L23" s="2"/>
@@ -44438,7 +44710,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R571be035568e463d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbf291451e3d4d08"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(register): record EVL-CHG-001 v0.4 approval and KT-STD-001 v1.12 entry
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/mvp-1-r1/98_work_progress/KenTender_Documentation_Control_Register.xlsx
+++ b/docs/mvp-1-r1/98_work_progress/KenTender_Documentation_Control_Register.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rddb14e0378f34914"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="2" r:id="Rf581a787ea874bcc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interfaces" sheetId="3" r:id="R5ef4927187344fab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="Raabcad47cdf6478d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery" sheetId="5" r:id="R0ce8146b9b3e41d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future Work" sheetId="6" r:id="Rda6ef2dd99354f21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="7" r:id="R3a6c9235a27649a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R24624d0ab4d84656"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documents" sheetId="2" r:id="Raf1e6a956a0c4a34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interfaces" sheetId="3" r:id="R639f3aeb3b154ee7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" r:id="R9816e5f1a98b4faf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery" sheetId="5" r:id="R63c1884036ce4839"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Future Work" sheetId="6" r:id="R892b2df5ec354432"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit" sheetId="7" r:id="R3a44bbb2b9654b03"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -153,7 +153,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="41">
+  <x:cellXfs count="42">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -272,6 +272,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="9" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1575,8 +1578,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DocumentsTable" displayName="DocumentsTable" ref="A5:P29" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:P29"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="DocumentsTable" displayName="DocumentsTable" ref="A5:P33" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="16">
     <x:tableColumn id="1" name="Document ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -1926,7 +1928,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="8" t="str">
-        <x:v>Current controlled baseline and delivery status as at 2026-09-28. Requirement approval, implementation, verification and release are tracked independently.</x:v>
+        <x:v>Current controlled baseline and delivery status as at 2026-09-30. Requirement approval, implementation, verification and release are tracked independently.</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -2050,17 +2052,17 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="20" t="n">
-        <x:f>COUNTA(Documents!A6:A32)</x:f>
-        <x:v>27</x:v>
+        <x:f>COUNTA(Documents!A6:A33)</x:f>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B6" s="20"/>
       <x:c r="C6" s="20" t="n">
-        <x:f>COUNTIF(Documents!F6:F32,"Approved requirement")</x:f>
-        <x:v>15</x:v>
+        <x:f>COUNTIF(Documents!F6:F33,"Approved requirement")</x:f>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D6" s="20"/>
       <x:c r="E6" s="20" t="n">
-        <x:f>COUNTIF(Documents!F6:F32,"Project Owner review")</x:f>
+        <x:f>COUNTIF(Documents!F6:F33,"Project Owner review")</x:f>
         <x:v>4</x:v>
       </x:c>
       <x:c r="F6" s="20"/>
@@ -8599,15 +8601,15 @@
       <x:c r="Y15" s="2"/>
       <x:c r="Z15" s="2"/>
     </x:row>
-    <x:row r="16" ht="44" customHeight="1">
-      <x:c r="A16" s="2" t="str">
+    <x:row r="16" ht="110" customHeight="1">
+      <x:c r="A16" s="24" t="str">
         <x:v>KT-STD-001</x:v>
       </x:c>
       <x:c r="B16" s="24" t="str">
         <x:v>Document, Design and Verification Standards</x:v>
       </x:c>
-      <x:c r="C16" s="2" t="str">
-        <x:v>1.10</x:v>
+      <x:c r="C16" s="24" t="str">
+        <x:v>1.12</x:v>
       </x:c>
       <x:c r="D16" s="24" t="str">
         <x:v>All</x:v>
@@ -8618,11 +8620,11 @@
       <x:c r="F16" s="24" t="str">
         <x:v>Approved requirement</x:v>
       </x:c>
-      <x:c r="G16" s="36" t="n">
-        <x:v>46294</x:v>
+      <x:c r="G16" s="41" t="n">
+        <x:v>46295</x:v>
       </x:c>
       <x:c r="H16" s="24" t="str">
-        <x:v>v1.9 approved 26 September 2026, retained as historical evidence</x:v>
+        <x:v>v1.11 and earlier</x:v>
       </x:c>
       <x:c r="I16" s="24" t="str">
         <x:v>Not applicable</x:v>
@@ -8633,20 +8635,20 @@
       <x:c r="K16" s="24" t="str">
         <x:v>Not applicable</x:v>
       </x:c>
-      <x:c r="L16" s="2" t="str">
+      <x:c r="L16" s="24" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="M16" s="24" t="str">
-        <x:v>Current cross-cutting standard, including plain language, minimum steps, Scheduled next step and actor/state/event conformance; retains earlier design and verification rules.</x:v>
+        <x:v>Current cross-cutting standard, including plain language, minimum steps, Scheduled next step and actor/state/event conformance; v1.11 adds the §8.3 fixture actors Daniel Otieno (technical operator) and Jane Wanjiku (public observer), and v1.12 adds Nadia Kamau (release operator); retains earlier design and verification rules.</x:v>
       </x:c>
       <x:c r="N16" s="24" t="str">
         <x:v>Workflow Guidance Standard; all controlled change documents</x:v>
       </x:c>
       <x:c r="O16" s="24" t="str">
-        <x:v>Apply approved v1.10 to future and revised design contracts: plain language, minimum steps, Scheduled next step and actor/state/event conformance.</x:v>
+        <x:v>Apply approved v1.12 to future and revised contracts; use its registered actors and retained design and verification rules.</x:v>
       </x:c>
       <x:c r="P16" s="24" t="str">
-        <x:v>https://chatgpt.com/api/library/files/libfile_17ffb496b8708191bfba06c99365e11c/download</x:v>
+        <x:v>https://chatgpt.com/api/library/files/libfile_4f7bf3bc8c0c8191b1e3ff2e2f3916da/download</x:v>
       </x:c>
       <x:c r="Q16" s="2"/>
       <x:c r="R16" s="2"/>
@@ -9581,23 +9583,55 @@
       <x:c r="Y32" s="2"/>
       <x:c r="Z32" s="2"/>
     </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="2"/>
-      <x:c r="B33" s="2"/>
-      <x:c r="C33" s="2"/>
-      <x:c r="D33" s="2"/>
-      <x:c r="E33" s="2"/>
-      <x:c r="F33" s="2"/>
-      <x:c r="G33" s="2"/>
-      <x:c r="H33" s="2"/>
-      <x:c r="I33" s="2"/>
-      <x:c r="J33" s="2"/>
-      <x:c r="K33" s="2"/>
-      <x:c r="L33" s="2"/>
-      <x:c r="M33" s="2"/>
-      <x:c r="N33" s="2"/>
-      <x:c r="O33" s="2"/>
-      <x:c r="P33" s="2"/>
+    <x:row r="33" ht="110" customHeight="1">
+      <x:c r="A33" s="24" t="str">
+        <x:v>EVL-CHG-001</x:v>
+      </x:c>
+      <x:c r="B33" s="24" t="str">
+        <x:v>Bid Evaluation</x:v>
+      </x:c>
+      <x:c r="C33" s="24" t="str">
+        <x:v>0.4</x:v>
+      </x:c>
+      <x:c r="D33" s="24" t="str">
+        <x:v>Bid Evaluation</x:v>
+      </x:c>
+      <x:c r="E33" s="24" t="str">
+        <x:v>Module requirements</x:v>
+      </x:c>
+      <x:c r="F33" s="24" t="str">
+        <x:v>Approved requirement</x:v>
+      </x:c>
+      <x:c r="G33" s="24" t="str">
+        <x:v>2026-09-30</x:v>
+      </x:c>
+      <x:c r="H33" s="24" t="str">
+        <x:v>v0.3 proposed detail; approved high-level automation approach retained</x:v>
+      </x:c>
+      <x:c r="I33" s="24" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="J33" s="24" t="str">
+        <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="K33" s="24" t="str">
+        <x:v>Not approved</x:v>
+      </x:c>
+      <x:c r="L33" s="24" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="M33" s="24" t="str">
+        <x:v>Automatic evaluation, focused committee review and signed report. Second-review corrections align commands, tasks, source issues, scope gates and dated fixtures.</x:v>
+      </x:c>
+      <x:c r="N33" s="24" t="str">
+        <x:v>KT-STD-001 v1.12; BOP v0.10; BDS v0.8; PRC v0.9; TRUST v0.1; TPR v0.13; STD-TPL v0.10. Coordinated owner-document amendments outstanding.</x:v>
+      </x:c>
+      <x:c r="O33" s="24" t="str">
+        <x:v>Implement approved v0.4 including R1–R3. Coordinate TPR publication binding, PRC, supplier correspondence and executable rules. Implementation and verification not started; Gate 1 unchanged.</x:v>
+      </x:c>
+      <x:c r="P33" s="24" t="str">
+        <x:v>https://chatgpt.com/api/library/files/libfile_afeac7a8387c81918c95b97accf8734e/download</x:v>
+      </x:c>
       <x:c r="Q33" s="2"/>
       <x:c r="R33" s="2"/>
       <x:c r="S33" s="2"/>
@@ -14336,7 +14370,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R44663dcb7900455e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5816d82678e541a2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20309,7 +20343,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R616750a2f016462e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8daba87739ce434f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26275,7 +26309,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b9767b4cdac4179"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc612c1b8f4454d3b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -32894,7 +32928,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R00da4d46689f4e68"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01909e40f84b4a97"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -38719,7 +38753,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R998d104da2ab441a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19d36bce9a674c5f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -44710,7 +44744,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcbf291451e3d4d08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82f269ba259c4e5b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs(kt-std): approve v1.13 (Evaluation fixture people)
Project Owner, 1 Oct 2026: "Approved".

- KT-STD-001 v1.13 marked approved: status, approval date and record,
  supersedes, approval effect (proposed wording retained) and version
  history. No other text changed.
- Register (yaml and workbook): KT-STD-001 at v1.13, approved 2026-10-01,
  proposed_revision cleared; the repository file is the approved text.
  EVL-CHG-001 notes the approval; SEED-OPS-001 depends on v1.13.
- FU-EVL-07 done.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/mvp-1-r1/98_work_progress/KenTender_Documentation_Control_Register.xlsx
+++ b/docs/mvp-1-r1/98_work_progress/KenTender_Documentation_Control_Register.xlsx
@@ -9298,7 +9298,7 @@
       </c>
       <c r="C16" s="24" t="inlineStr">
         <is>
-          <t>1.12</t>
+          <t>1.13</t>
         </is>
       </c>
       <c r="D16" s="24" t="inlineStr">
@@ -9317,11 +9317,11 @@
         </is>
       </c>
       <c r="G16" s="50" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="H16" s="24" t="inlineStr">
         <is>
-          <t>v1.11 and earlier</t>
+          <t>v1.12 and earlier</t>
         </is>
       </c>
       <c r="I16" s="24" t="inlineStr">
@@ -9346,7 +9346,7 @@
       </c>
       <c r="M16" s="24" t="inlineStr">
         <is>
-          <t>Current cross-cutting standard, including plain language, minimum steps, Scheduled next step and actor/state/event conformance; v1.11 adds the §8.3 fixture actors Daniel Otieno (technical operator) and Jane Wanjiku (public observer), and v1.12 adds Nadia Kamau (release operator); retains earlier design and verification rules.</t>
+          <t>Current cross-cutting standard, including plain language, minimum steps, Scheduled next step and actor/state/event conformance; v1.11 adds the §8.3 fixture actors Daniel Otieno (technical operator) and Jane Wanjiku (public observer), and v1.12 adds Nadia Kamau (release operator); retains earlier design and verification rules. v1.13 adds the Evaluation fixture actors Grace Wambui, Peter Mugo, Ruth Achieng and Esther Njeri, and Brian Wafula's separately appointed secretary capacity.</t>
         </is>
       </c>
       <c r="N16" s="24" t="inlineStr">
@@ -9356,12 +9356,12 @@
       </c>
       <c r="O16" s="24" t="inlineStr">
         <is>
-          <t>Review proposed v1.13: register Evaluation actors and Brian’s separate secretary capacity. No automatic appointment or expanded support access. Approved v1.12 retained.</t>
+          <t>Apply approved v1.13 (Project Owner, 2026-10-01: "Approved") to future and revised contracts; use its registered actors. The repository file is the approved text: it adds the 2026-10-01 rewording of "For TND-MOH-2027-033" as an example of the generated reference (DEC-027) and names Esther Njeri's Evaluation Technical Support responsibility, beyond the library draft.</t>
         </is>
       </c>
       <c r="P16" s="24" t="inlineStr">
         <is>
-          <t>https://chatgpt.com/api/library/files/libfile_4f7bf3bc8c0c8191b1e3ff2e2f3916da/download</t>
+          <t>https://chatgpt.com/api/library/files/libfile_67c97b311d088191b90d070526a4bfbc/download</t>
         </is>
       </c>
       <c r="Q16" s="2" t="n"/>
@@ -10832,7 +10832,7 @@
       </c>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>Approved EVL v0.4 retained. Four coordinated owner successors drafted and linked in their register entries. Review amendments and implement/test the bindings; executable template rules and legal/Trust work remain open. Gate 1 unchanged.</t>
+          <t>Approved EVL v0.4 retained. Four coordinated owner successors drafted and linked in their register entries. Review amendments and implement/test the bindings; executable template rules and legal/Trust work remain open. Gate 1 unchanged. KT-STD-001 v1.13 approved 2026-10-01.</t>
         </is>
       </c>
       <c r="P33" s="24" t="inlineStr">
@@ -11003,7 +11003,7 @@
       </c>
       <c r="N35" s="24" t="inlineStr">
         <is>
-          <t>KT-STD-001 v1.12; SEED-001 v1.3; the module documents each stage cites in its §2</t>
+          <t>KT-STD-001 v1.13; SEED-001 v1.3; the module documents each stage cites in its §2</t>
         </is>
       </c>
       <c r="O35" s="24" t="inlineStr">

</xml_diff>